<commit_message>
Add the Excel walkthrough PDF and update the model after the first Solver run
</commit_message>
<xml_diff>
--- a/excel/budget_model.xlsx
+++ b/excel/budget_model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40576ae3754c8ac9/Υπολογιστής/Ο Φάκελός μου/Data analyst projects/FinTech Customer Acquisition and Profitability Analysis/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{DA684D4A-D9C9-4D3B-8B67-0B4778129DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3B2653E-D43B-4A4F-87F6-335E28E63077}"/>
+  <xr:revisionPtr revIDLastSave="338" documentId="8_{DA684D4A-D9C9-4D3B-8B67-0B4778129DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED350CFD-074E-47C8-B8FC-68AE026DAD2F}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -25,26 +25,26 @@
     <sheet name="Data_Curve" sheetId="10" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="solver_adj" localSheetId="4">Optimizer!$E$5:$E$8</definedName>
-    <definedName name="solver_eng" localSheetId="4">1</definedName>
+    <definedName name="solver_adj" localSheetId="4" hidden="1">Optimizer!$E$5:$E$8</definedName>
+    <definedName name="solver_eng" localSheetId="4" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="4">1</definedName>
-    <definedName name="solver_lhs1" localSheetId="4">Optimizer!$E$5:$E$8</definedName>
-    <definedName name="solver_lhs2" localSheetId="4">Optimizer!$E$5:$E$8</definedName>
-    <definedName name="solver_lhs3" localSheetId="4">Optimizer!$E$9</definedName>
+    <definedName name="solver_lhs1" localSheetId="4" hidden="1">Optimizer!$E$5:$E$8</definedName>
+    <definedName name="solver_lhs2" localSheetId="4" hidden="1">Optimizer!$E$5:$E$8</definedName>
+    <definedName name="solver_lhs3" localSheetId="4" hidden="1">Optimizer!$E$9</definedName>
     <definedName name="solver_lin" localSheetId="4">2</definedName>
-    <definedName name="solver_neg" localSheetId="4">1</definedName>
-    <definedName name="solver_num" localSheetId="4">3</definedName>
+    <definedName name="solver_neg" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_num" localSheetId="4" hidden="1">3</definedName>
     <definedName name="solver_nwt" localSheetId="4">1</definedName>
-    <definedName name="solver_opt" localSheetId="4">Optimizer!$B$14</definedName>
-    <definedName name="solver_rel1" localSheetId="4">3</definedName>
-    <definedName name="solver_rel2" localSheetId="4">1</definedName>
-    <definedName name="solver_rel3" localSheetId="4">1</definedName>
-    <definedName name="solver_rhs1" localSheetId="4">Optimizer!$C$5:$C$8</definedName>
-    <definedName name="solver_rhs2" localSheetId="4">Optimizer!$D$5:$D$8</definedName>
-    <definedName name="solver_rhs3" localSheetId="4">Optimizer!$B$11</definedName>
-    <definedName name="solver_typ" localSheetId="4">1</definedName>
-    <definedName name="solver_val" localSheetId="4">0</definedName>
-    <definedName name="solver_ver" localSheetId="4">3</definedName>
+    <definedName name="solver_opt" localSheetId="4" hidden="1">Optimizer!$B$14</definedName>
+    <definedName name="solver_rel1" localSheetId="4" hidden="1">3</definedName>
+    <definedName name="solver_rel2" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_rhs1" localSheetId="4" hidden="1">Optimizer!$C$5:$C$8</definedName>
+    <definedName name="solver_rhs2" localSheetId="4" hidden="1">Optimizer!$D$5:$D$8</definedName>
+    <definedName name="solver_rhs3" localSheetId="4" hidden="1">Optimizer!$B$11</definedName>
+    <definedName name="solver_typ" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_val" localSheetId="4" hidden="1">0</definedName>
+    <definedName name="solver_ver" localSheetId="4" hidden="1">3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -916,6 +916,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:rPr lang="en-US"/>
               <a:t>Cumulative margin per customer by month</a:t>
             </a:r>
           </a:p>
@@ -1513,6 +1514,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
+                  <a:rPr lang="en-US"/>
                   <a:t>Month since first deposit</a:t>
                 </a:r>
               </a:p>
@@ -1549,6 +1551,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
+                  <a:rPr lang="en-US"/>
                   <a:t>EUR per customer</a:t>
                 </a:r>
               </a:p>
@@ -1598,6 +1601,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:rPr lang="en-US"/>
               <a:t>Spend by channel: baseline vs recommended (EUR, quarter)</a:t>
             </a:r>
           </a:p>
@@ -1710,16 +1714,16 @@
                 <c:formatCode>#,##0;\(#,##0\);\-</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>1558.24</c:v>
+                  <c:v>1558.2399999999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2687.39</c:v>
+                  <c:v>2687.395</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>9515.0400000000009</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1297.6099999999999</c:v>
+                  <c:v>1297.6079999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1778,6 +1782,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
+                  <a:rPr lang="en-US"/>
                   <a:t>EUR per quarter</a:t>
                 </a:r>
               </a:p>
@@ -1880,6 +1885,10 @@
     <xdr:clientData/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2238,7 +2247,7 @@
       </c>
       <c r="C9" s="8">
         <f>Optimizer!E5</f>
-        <v>1558.24</v>
+        <v>1558.2399999999998</v>
       </c>
       <c r="D9" s="9">
         <f>Optimizer!F5</f>
@@ -2268,11 +2277,11 @@
       </c>
       <c r="C10" s="8">
         <f>Optimizer!E6</f>
-        <v>2687.39</v>
+        <v>2687.395</v>
       </c>
       <c r="D10" s="9">
         <f>Optimizer!F6</f>
-        <v>-0.50000093026890358</v>
+        <v>-0.5</v>
       </c>
       <c r="E10" s="10">
         <f>ROUND(C10/100,0)*100</f>
@@ -2328,11 +2337,11 @@
       </c>
       <c r="C12" s="8">
         <f>Optimizer!E8</f>
-        <v>1297.6099999999999</v>
+        <v>1297.6079999999999</v>
       </c>
       <c r="D12" s="9">
         <f>Optimizer!F8</f>
-        <v>0.20000184955703104</v>
+        <v>0.19999999999999996</v>
       </c>
       <c r="E12" s="10">
         <f>ROUND(C12/100,0)*100</f>
@@ -2357,11 +2366,11 @@
       </c>
       <c r="C13" s="13">
         <f>Optimizer!E9</f>
-        <v>15058.280000000002</v>
+        <v>15058.283000000001</v>
       </c>
       <c r="D13" s="14">
         <f>Optimizer!F9</f>
-        <v>-0.4735362303335805</v>
+        <v>-0.47353612544834067</v>
       </c>
       <c r="E13" s="13">
         <f>SUM(E9:E12)</f>
@@ -2390,7 +2399,7 @@
       </c>
       <c r="B17" s="7">
         <f>Optimizer!B14</f>
-        <v>-56843.197213699066</v>
+        <v>-56843.210383740414</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -2399,7 +2408,7 @@
       </c>
       <c r="B18" s="16">
         <f>Optimizer!B15</f>
-        <v>40720.443804187758</v>
+        <v>40720.430634146411</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
@@ -5477,7 +5486,7 @@
         <v>4674.72</v>
       </c>
       <c r="E5" s="38">
-        <v>1558.24</v>
+        <v>1558.2399999999998</v>
       </c>
       <c r="F5" s="39">
         <f>E5/B5-1</f>
@@ -5521,11 +5530,11 @@
         <v>8062.1849999999995</v>
       </c>
       <c r="E6" s="38">
-        <v>2687.39</v>
+        <v>2687.395</v>
       </c>
       <c r="F6" s="39">
         <f>E6/B6-1</f>
-        <v>-0.50000093026890358</v>
+        <v>-0.5</v>
       </c>
       <c r="G6" s="37">
         <f>Assumptions!$B$6*Curves!E6*(B6/Assumptions!$B$6)^Curves!C6</f>
@@ -5533,7 +5542,7 @@
       </c>
       <c r="H6" s="37">
         <f>Assumptions!$B$6*Curves!E6*(E6/Assumptions!$B$6)^Curves!C6</f>
-        <v>140.65828770463119</v>
+        <v>140.65846862866036</v>
       </c>
       <c r="I6" s="11">
         <f>INDEX(Unit_Economics!$T$5:$T$9,MATCH(A6,Unit_Economics!$A$5:$A$9,0))</f>
@@ -5545,7 +5554,7 @@
       </c>
       <c r="K6" s="10">
         <f>H6*I6</f>
-        <v>-4970.217496644962</v>
+        <v>-4970.2238896687222</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -5609,11 +5618,11 @@
         <v>1297.6079999999999</v>
       </c>
       <c r="E8" s="38">
-        <v>1297.6099999999999</v>
+        <v>1297.6079999999999</v>
       </c>
       <c r="F8" s="39">
         <f>E8/B8-1</f>
-        <v>0.20000184955703104</v>
+        <v>0.19999999999999996</v>
       </c>
       <c r="G8" s="37">
         <f>Assumptions!$B$6*Curves!E8*(B8/Assumptions!$B$6)^Curves!C8</f>
@@ -5621,7 +5630,7 @@
       </c>
       <c r="H8" s="37">
         <f>Assumptions!$B$6*Curves!E8*(E8/Assumptions!$B$6)^Curves!C8</f>
-        <v>115.44831203492785</v>
+        <v>115.44823882568373</v>
       </c>
       <c r="I8" s="11">
         <f>INDEX(Unit_Economics!$T$5:$T$9,MATCH(A8,Unit_Economics!$A$5:$A$9,0))</f>
@@ -5633,7 +5642,7 @@
       </c>
       <c r="K8" s="10">
         <f>H8*I8</f>
-        <v>5956.2191992132857</v>
+        <v>5956.2154221956953</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
@@ -5648,11 +5657,11 @@
       <c r="D9" s="15"/>
       <c r="E9" s="13">
         <f>SUM(E5:E8)</f>
-        <v>15058.280000000002</v>
+        <v>15058.283000000001</v>
       </c>
       <c r="F9" s="14">
         <f>E9/B9-1</f>
-        <v>-0.4735362303335805</v>
+        <v>-0.47353612544834067</v>
       </c>
       <c r="G9" s="40">
         <f>SUM(G5:G8)</f>
@@ -5660,7 +5669,7 @@
       </c>
       <c r="H9" s="40">
         <f>SUM(H5:H8)</f>
-        <v>470.02351237207495</v>
+        <v>470.02362008685992</v>
       </c>
       <c r="I9" s="15"/>
       <c r="J9" s="13">
@@ -5669,7 +5678,7 @@
       </c>
       <c r="K9" s="13">
         <f>SUM(K5:K8)</f>
-        <v>-41784.917213699067</v>
+        <v>-41784.927383740411</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
@@ -5687,7 +5696,7 @@
       </c>
       <c r="B12" s="10">
         <f>E9</f>
-        <v>15058.280000000002</v>
+        <v>15058.283000000001</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -5705,7 +5714,7 @@
       </c>
       <c r="B14" s="16">
         <f>K9-E9</f>
-        <v>-56843.197213699066</v>
+        <v>-56843.210383740414</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
@@ -5714,7 +5723,7 @@
       </c>
       <c r="B15" s="13">
         <f>B14-B13</f>
-        <v>40720.443804187758</v>
+        <v>40720.430634146411</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
@@ -5852,14 +5861,14 @@
         <v>470</v>
       </c>
       <c r="J5" s="10">
-        <v>-56843</v>
+        <v>-56843.21</v>
       </c>
       <c r="K5" s="10">
-        <v>-97564</v>
+        <v>-97563.64</v>
       </c>
       <c r="L5" s="43">
         <f t="shared" ref="L5:L12" si="1">J5-K5</f>
-        <v>40721</v>
+        <v>40720.43</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -5892,14 +5901,14 @@
         <v>470</v>
       </c>
       <c r="J6" s="10">
-        <v>-56843</v>
+        <v>-56843.21</v>
       </c>
       <c r="K6" s="10">
-        <v>-97564</v>
+        <v>-97563.64</v>
       </c>
       <c r="L6" s="43">
         <f t="shared" si="1"/>
-        <v>40721</v>
+        <v>40720.43</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -5932,14 +5941,14 @@
         <v>470</v>
       </c>
       <c r="J7" s="10">
-        <v>-56843</v>
+        <v>-56843.21</v>
       </c>
       <c r="K7" s="10">
-        <v>-97564</v>
+        <v>-97563.64</v>
       </c>
       <c r="L7" s="43">
         <f t="shared" si="1"/>
-        <v>40721</v>
+        <v>40720.43</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -5972,14 +5981,14 @@
         <v>460</v>
       </c>
       <c r="J8" s="10">
-        <v>-88648</v>
+        <v>-88647.74</v>
       </c>
       <c r="K8" s="10">
-        <v>-145370</v>
+        <v>-145369.99</v>
       </c>
       <c r="L8" s="43">
         <f t="shared" si="1"/>
-        <v>56722</v>
+        <v>56722.249999999985</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -6012,14 +6021,14 @@
         <v>470</v>
       </c>
       <c r="J9" s="10">
-        <v>-25021</v>
+        <v>-25020.92</v>
       </c>
       <c r="K9" s="10">
-        <v>-49757</v>
+        <v>-49757.3</v>
       </c>
       <c r="L9" s="43">
         <f t="shared" si="1"/>
-        <v>24736</v>
+        <v>24736.380000000005</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -6052,14 +6061,14 @@
         <v>448</v>
       </c>
       <c r="J10" s="10">
-        <v>-55514</v>
+        <v>-55514.3</v>
       </c>
       <c r="K10" s="10">
-        <v>-92832</v>
+        <v>-92832.03</v>
       </c>
       <c r="L10" s="43">
         <f t="shared" si="1"/>
-        <v>37318</v>
+        <v>37317.729999999996</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -6092,14 +6101,14 @@
         <v>470</v>
       </c>
       <c r="J11" s="10">
-        <v>-32595</v>
+        <v>-32595.19</v>
       </c>
       <c r="K11" s="10">
-        <v>-62702</v>
+        <v>-62702.22</v>
       </c>
       <c r="L11" s="43">
         <f t="shared" si="1"/>
-        <v>30107</v>
+        <v>30107.030000000002</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -6132,14 +6141,14 @@
         <v>572</v>
       </c>
       <c r="J12" s="10">
-        <v>-75921</v>
+        <v>-75920.679999999993</v>
       </c>
       <c r="K12" s="10">
-        <v>-97564</v>
+        <v>-97563.64</v>
       </c>
       <c r="L12" s="43">
         <f t="shared" si="1"/>
-        <v>21643</v>
+        <v>21642.960000000006</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Add LTV scenarios to the Excel model and re-run the optimizer for each
</commit_message>
<xml_diff>
--- a/excel/budget_model.xlsx
+++ b/excel/budget_model.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40576ae3754c8ac9/Υπολογιστής/Ο Φάκελός μου/Data analyst projects/FinTech Customer Acquisition and Profitability Analysis/excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40576ae3754c8ac9/Υπολογιστής/Ο Φάκελός μου/Data analyst projects/FinTech Customer Acquisition and Profitability Analysis/FinTech-Customer-Acquisition-and-Profitability-Analysis/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="429" documentId="8_{DA684D4A-D9C9-4D3B-8B67-0B4778129DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30A4A347-BCB6-4D42-9443-E0871C1CE755}"/>
+  <xr:revisionPtr revIDLastSave="3986" documentId="8_{DA684D4A-D9C9-4D3B-8B67-0B4778129DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3F7502A0-37FF-471B-BEB2-74E437448CCE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,11 +19,16 @@
     <sheet name="Curves" sheetId="4" r:id="rId4"/>
     <sheet name="Optimizer" sheetId="5" r:id="rId5"/>
     <sheet name="Scenarios" sheetId="6" r:id="rId6"/>
-    <sheet name="Pivot_Tables" sheetId="12" r:id="rId7"/>
-    <sheet name="Notes" sheetId="7" r:id="rId8"/>
-    <sheet name="Data_Scorecard" sheetId="8" r:id="rId9"/>
-    <sheet name="Data_Monthly" sheetId="9" r:id="rId10"/>
-    <sheet name="Data_Curve" sheetId="10" r:id="rId11"/>
+    <sheet name="LTV_Scenarios" sheetId="18" r:id="rId7"/>
+    <sheet name="Sheet4" sheetId="17" r:id="rId8"/>
+    <sheet name="Sheet3" sheetId="16" r:id="rId9"/>
+    <sheet name="Sheet2" sheetId="15" r:id="rId10"/>
+    <sheet name="Sheet1" sheetId="14" r:id="rId11"/>
+    <sheet name="Pivot_Tables" sheetId="12" r:id="rId12"/>
+    <sheet name="Notes" sheetId="7" r:id="rId13"/>
+    <sheet name="Data_Scorecard" sheetId="8" r:id="rId14"/>
+    <sheet name="Data_Monthly" sheetId="9" r:id="rId15"/>
+    <sheet name="Data_Curve" sheetId="10" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="solver_adj" localSheetId="4" hidden="1">Optimizer!$E$5:$E$8</definedName>
@@ -49,7 +54,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId12"/>
+    <pivotCache cacheId="0" r:id="rId17"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -68,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="251">
   <si>
     <t>Budget model: which channels deserve next quarter's marketing budget?</t>
   </si>
@@ -755,6 +760,72 @@
   </si>
   <si>
     <t>Pivot tables: spend, customers and cost per customer by quarter and channel</t>
+  </si>
+  <si>
+    <t>LTV scenario shift (added to the risk-adjusted LTV)</t>
+  </si>
+  <si>
+    <t>Active shift (EUR per customer)</t>
+  </si>
+  <si>
+    <t>Pessimistic shift</t>
+  </si>
+  <si>
+    <t>Default 0 = point estimates, as delivered. Columns C and D are the low and high end of the 95% bootstrap interval of each channel risk-adjusted LTV, minus its point estimate (python/results/ltv_bootstrap.csv). To test a scenario, copy column C or D into column B, then run Solver on the Optimizer sheet. Sheet LTV_Scenarios holds the results.</t>
+  </si>
+  <si>
+    <t>LTV scenarios</t>
+  </si>
+  <si>
+    <t>The risk-adjusted LTV of each channel is moved to the low or high end of its 95% bootstrap interval (shift in Assumptions, rows 27 to 31). Each row is the Solver optimum for that case (pasted values).</t>
+  </si>
+  <si>
+    <t>What changes</t>
+  </si>
+  <si>
+    <t>Shift affiliate (EUR)</t>
+  </si>
+  <si>
+    <t>Shift paid_search (EUR)</t>
+  </si>
+  <si>
+    <t>Shift paid_social (EUR)</t>
+  </si>
+  <si>
+    <t>Shift referral (EUR)</t>
+  </si>
+  <si>
+    <t>Point estimates, as delivered</t>
+  </si>
+  <si>
+    <t>Pessimistic</t>
+  </si>
+  <si>
+    <t>Every channel at the low end of its 95% interval</t>
+  </si>
+  <si>
+    <t>Optimistic</t>
+  </si>
+  <si>
+    <t>Every channel at the high end of its 95% interval</t>
+  </si>
+  <si>
+    <t>Referral weak, others strong</t>
+  </si>
+  <si>
+    <t>Referral at its low end, all others at their high end</t>
+  </si>
+  <si>
+    <t>Referral strong, others weak</t>
+  </si>
+  <si>
+    <t>Referral at its high end, all others at their low end</t>
+  </si>
+  <si>
+    <t>Optimistic shift</t>
+  </si>
+  <si>
+    <t>Reading: affiliate and paid social stay at their lower limit in all five cases, even when their value is at the high end of its interval, so cutting them does not depend on the point estimates. Referral and paid search are the two swing channels: referral falls to its lower limit when its value is at the low end (the interval includes zero), and paid search rises to its upper limit when its value is at the high end. Net profit stays negative in every case, and the uplift is positive in every case.</t>
   </si>
 </sst>
 </file>
@@ -771,7 +842,7 @@
     <numFmt numFmtId="170" formatCode="0.000"/>
     <numFmt numFmtId="171" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -858,6 +929,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -882,7 +966,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -1016,11 +1100,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1109,13 +1202,6 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1146,14 +1232,47 @@
     </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="2" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="33">
+  <dxfs count="49">
     <dxf>
       <font>
-        <b/>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -1163,17 +1282,11 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
+        <color auto="1"/>
         <name val="Arial"/>
         <scheme val="none"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF1F3864"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color rgb="FFBFBFBF"/>
@@ -1181,8 +1294,12 @@
         <right style="thin">
           <color rgb="FFBFBFBF"/>
         </right>
-        <top/>
-        <bottom/>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1201,6 +1318,444 @@
         <name val="Arial"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE2EFDA"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1621,22 +2176,39 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
         <bottom style="thin">
           <color rgb="FFBFBFBF"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
       <border outline="0">
-        <left style="thin">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
         <bottom style="thin">
           <color rgb="FFBFBFBF"/>
         </bottom>
@@ -1675,23 +2247,6 @@
         <top/>
         <bottom/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -2077,25 +2632,76 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
         <bottom style="thin">
           <color rgb="FFBFBFBF"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
       <border outline="0">
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF1F3864"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color rgb="FFBFBFBF"/>
         </left>
         <right style="thin">
           <color rgb="FFBFBFBF"/>
         </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
   </dxfs>
@@ -3707,6 +4313,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
       <x14:pivotCacheDefinition/>
+    </ext>
+    <ext xmlns:xlpdsc="http://schemas.microsoft.com/office/spreadsheetml/2026/pivotDataSourceClean" uri="{F4336242-56EE-4DD3-A5F7-E900642BF6E9}">
+      <xlpdsc:dataSourceClean>1</xlpdsc:dataSourceClean>
     </ext>
   </extLst>
 </pivotCacheDefinition>
@@ -4678,6 +5287,208 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A6B9975A-04F5-4C52-B5DD-F27FC6E13B4C}" name="pt_customers" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A19:F29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField axis="axisCol" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="165" showAll="0"/>
+    <pivotField dataField="1" numFmtId="2" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="9">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="9">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="0"/>
+  </colFields>
+  <colItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Customers" fld="3" baseField="0" baseItem="0" numFmtId="3"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleMedium2" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EEB6DEEC-373F-4F73-9BA5-F336E9ED42DE}" name="pt_spend" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A5:F15" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField axis="axisCol" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField dataField="1" numFmtId="165" showAll="0"/>
+    <pivotField numFmtId="2" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="9">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="9">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="0"/>
+  </colFields>
+  <colItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Ad spend" fld="2" baseField="0" baseItem="0" numFmtId="3"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleMedium2" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{94AC0DEC-182A-4E90-B978-16061F2A19B4}" name="pt_cost" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A33:F43" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -4828,210 +5639,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A6B9975A-04F5-4C52-B5DD-F27FC6E13B4C}" name="pt_customers" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A19:F29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField axis="axisCol" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="165" showAll="0"/>
-    <pivotField dataField="1" numFmtId="2" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="9">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="7"/>
-  </rowFields>
-  <rowItems count="9">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="0"/>
-  </colFields>
-  <colItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Customers" fld="3" baseField="0" baseItem="0" numFmtId="3"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleMedium2" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EEB6DEEC-373F-4F73-9BA5-F336E9ED42DE}" name="pt_spend" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A5:F15" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField axis="axisCol" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField dataField="1" numFmtId="165" showAll="0"/>
-    <pivotField numFmtId="2" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="9">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="7"/>
-  </rowFields>
-  <rowItems count="9">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="0"/>
-  </colFields>
-  <colItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Ad spend" fld="2" baseField="0" baseItem="0" numFmtId="3"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleMedium2" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AC8DC09A-E2BB-48D4-87FC-A004F9136AB4}" name="tblAllocation" displayName="tblAllocation" ref="A4:K8" totalsRowShown="0" headerRowDxfId="17" dataDxfId="18" headerRowBorderDxfId="31" tableBorderDxfId="32" totalsRowBorderDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AC8DC09A-E2BB-48D4-87FC-A004F9136AB4}" name="tblAllocation" displayName="tblAllocation" ref="A4:K8" totalsRowShown="0" headerRowDxfId="48" dataDxfId="46" headerRowBorderDxfId="47" tableBorderDxfId="45" totalsRowBorderDxfId="44">
   <autoFilter ref="A4:K8" xr:uid="{AC8DC09A-E2BB-48D4-87FC-A004F9136AB4}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -5046,33 +5655,33 @@
     <filterColumn colId="10" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{90ACE40C-34FF-4344-8F5B-3C122A8EB768}" name="Channel" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{CFF5D8CE-4F2B-4CBD-81F5-19DB86D32687}" name="Baseline spend, Jul to Sep 2026 (EUR)" dataDxfId="28">
+    <tableColumn id="1" xr3:uid="{90ACE40C-34FF-4344-8F5B-3C122A8EB768}" name="Channel" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{CFF5D8CE-4F2B-4CBD-81F5-19DB86D32687}" name="Baseline spend, Jul to Sep 2026 (EUR)" dataDxfId="42">
       <calculatedColumnFormula>SUMIFS(Data_Monthly!$C$2:$C$97,Data_Monthly!$A$2:$A$97,A5,Data_Monthly!$E$2:$E$97,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{C73D6A21-26F1-455B-B3CE-0C78461D1ADE}" name="Lower limit (EUR)" dataDxfId="27">
+    <tableColumn id="3" xr3:uid="{C73D6A21-26F1-455B-B3CE-0C78461D1ADE}" name="Lower limit (EUR)" dataDxfId="41">
       <calculatedColumnFormula>B5*Assumptions!$B$9</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{E77E3CCE-452A-4EC3-94FF-A836CDEBA5FC}" name="Upper limit (EUR)" dataDxfId="26">
+    <tableColumn id="4" xr3:uid="{E77E3CCE-452A-4EC3-94FF-A836CDEBA5FC}" name="Upper limit (EUR)" dataDxfId="40">
       <calculatedColumnFormula>B5*IF(A5="referral",Assumptions!$B$11,Assumptions!$B$10)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{8786FC5F-5E15-4932-9660-0500AC9E8F67}" name="Recommended spend (EUR)  &lt;- Solver changes these" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{CE1A2D8E-82D2-49DA-B043-CD145336C6EB}" name="Change vs baseline" dataDxfId="24">
+    <tableColumn id="5" xr3:uid="{8786FC5F-5E15-4932-9660-0500AC9E8F67}" name="Recommended spend (EUR)  &lt;- Solver changes these" dataDxfId="39"/>
+    <tableColumn id="6" xr3:uid="{CE1A2D8E-82D2-49DA-B043-CD145336C6EB}" name="Change vs baseline" dataDxfId="38">
       <calculatedColumnFormula>E5/B5-1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{5DB595EB-952F-4BFD-93FA-F986406C4D62}" name="Customers at baseline spend" dataDxfId="23">
+    <tableColumn id="7" xr3:uid="{5DB595EB-952F-4BFD-93FA-F986406C4D62}" name="Customers at baseline spend" dataDxfId="37">
       <calculatedColumnFormula>Assumptions!$B$6*Curves!E5*(B5/Assumptions!$B$6)^Curves!C5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{13AC6CD4-6A69-42F1-8D13-BD9DB5A42602}" name="Customers at recommended spend" dataDxfId="22">
+    <tableColumn id="8" xr3:uid="{13AC6CD4-6A69-42F1-8D13-BD9DB5A42602}" name="Customers at recommended spend" dataDxfId="36">
       <calculatedColumnFormula>Assumptions!$B$6*Curves!E5*(E5/Assumptions!$B$6)^Curves!C5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{041B4720-C84E-45B9-ADE2-8BEBF0DFCBD0}" name="Net value per customer (EUR)" dataDxfId="21">
+    <tableColumn id="9" xr3:uid="{041B4720-C84E-45B9-ADE2-8BEBF0DFCBD0}" name="Net value per customer (EUR)" dataDxfId="35">
       <calculatedColumnFormula>VLOOKUP(A5,Unit_Economics!$A$5:$T$9,20,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{66919F9C-3E7B-46B1-9653-A59A09C73B58}" name="Value of customers, baseline (EUR)" dataDxfId="20">
+    <tableColumn id="10" xr3:uid="{66919F9C-3E7B-46B1-9653-A59A09C73B58}" name="Value of customers, baseline (EUR)" dataDxfId="34">
       <calculatedColumnFormula>G5*I5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{FB5F8EA3-E836-4712-A5D0-940FDF8E3D29}" name="Value of customers, recommended (EUR)" dataDxfId="19">
+    <tableColumn id="11" xr3:uid="{FB5F8EA3-E836-4712-A5D0-940FDF8E3D29}" name="Value of customers, recommended (EUR)" dataDxfId="33">
       <calculatedColumnFormula>H5*I5</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5081,7 +5690,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E837F1CC-31FE-4B5C-A277-85EAD6FD0B38}" name="tblScenarios" displayName="tblScenarios" ref="A4:L12" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1" headerRowBorderDxfId="15" tableBorderDxfId="16" totalsRowBorderDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E837F1CC-31FE-4B5C-A277-85EAD6FD0B38}" name="tblScenarios" displayName="tblScenarios" ref="A4:L12" totalsRowShown="0" headerRowDxfId="32" dataDxfId="30" headerRowBorderDxfId="31" tableBorderDxfId="29" totalsRowBorderDxfId="28">
   <autoFilter ref="A4:L12" xr:uid="{E837F1CC-31FE-4B5C-A277-85EAD6FD0B38}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -5097,21 +5706,67 @@
     <filterColumn colId="11" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{379ED11E-2D94-4211-8842-6FBE97A8EE58}" name="Scenario" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{B35D69D6-B058-4058-9180-A3A8A4189631}" name="Lever" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{C1DD03A6-4712-4A39-BD8E-92B2EA3E2EA0}" name="Budget ceiling (EUR)" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{CD80F512-FDFD-43AD-8386-81DB6E731717}" name="affiliate spend (EUR)" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{045B13DD-7FAE-49D7-919F-1B6482A85DCC}" name="paid_search spend (EUR)" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{837CDB58-80E5-4A80-8446-9BDF569D0A47}" name="paid_social spend (EUR)" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{94A228FC-48CE-41E1-9F30-2D3B74A7241B}" name="referral spend (EUR)" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{40229F94-C4C0-4AA1-B323-59F713BD5D0D}" name="Total spend (EUR)" dataDxfId="6">
+    <tableColumn id="1" xr3:uid="{379ED11E-2D94-4211-8842-6FBE97A8EE58}" name="Scenario" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{B35D69D6-B058-4058-9180-A3A8A4189631}" name="Lever" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{C1DD03A6-4712-4A39-BD8E-92B2EA3E2EA0}" name="Budget ceiling (EUR)" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{CD80F512-FDFD-43AD-8386-81DB6E731717}" name="affiliate spend (EUR)" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{045B13DD-7FAE-49D7-919F-1B6482A85DCC}" name="paid_search spend (EUR)" dataDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{837CDB58-80E5-4A80-8446-9BDF569D0A47}" name="paid_social spend (EUR)" dataDxfId="22"/>
+    <tableColumn id="7" xr3:uid="{94A228FC-48CE-41E1-9F30-2D3B74A7241B}" name="referral spend (EUR)" dataDxfId="21"/>
+    <tableColumn id="8" xr3:uid="{40229F94-C4C0-4AA1-B323-59F713BD5D0D}" name="Total spend (EUR)" dataDxfId="20">
       <calculatedColumnFormula>SUM(D5:G5)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{8A906FA2-888B-466B-8E51-63BEFC57350E}" name="Customers won" dataDxfId="5"/>
-    <tableColumn id="10" xr3:uid="{FEB89709-AC45-4A0D-A707-16FD375A5B60}" name="Net profit at recommended spend (EUR)" dataDxfId="4"/>
-    <tableColumn id="11" xr3:uid="{1A136D42-B00E-43EF-A368-6196D78A78D0}" name="Net profit at baseline spend (EUR)" dataDxfId="3"/>
-    <tableColumn id="12" xr3:uid="{BBB830FB-593F-4760-81CB-B29AFD974D95}" name="Uplift (EUR)" dataDxfId="2">
+    <tableColumn id="9" xr3:uid="{8A906FA2-888B-466B-8E51-63BEFC57350E}" name="Customers won" dataDxfId="19"/>
+    <tableColumn id="10" xr3:uid="{FEB89709-AC45-4A0D-A707-16FD375A5B60}" name="Net profit at recommended spend (EUR)" dataDxfId="18"/>
+    <tableColumn id="11" xr3:uid="{1A136D42-B00E-43EF-A368-6196D78A78D0}" name="Net profit at baseline spend (EUR)" dataDxfId="17"/>
+    <tableColumn id="12" xr3:uid="{BBB830FB-593F-4760-81CB-B29AFD974D95}" name="Uplift (EUR)" dataDxfId="16">
       <calculatedColumnFormula>J5-K5</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D58DFAFE-0A67-42D2-B83A-C56A872441F7}" name="tblLtvScenarios" displayName="tblLtvScenarios" ref="A4:O9" totalsRowShown="0" headerRowDxfId="15">
+  <autoFilter ref="A4:O9" xr:uid="{D58DFAFE-0A67-42D2-B83A-C56A872441F7}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
+    <filterColumn colId="7" hiddenButton="1"/>
+    <filterColumn colId="8" hiddenButton="1"/>
+    <filterColumn colId="9" hiddenButton="1"/>
+    <filterColumn colId="10" hiddenButton="1"/>
+    <filterColumn colId="11" hiddenButton="1"/>
+    <filterColumn colId="12" hiddenButton="1"/>
+    <filterColumn colId="13" hiddenButton="1"/>
+    <filterColumn colId="14" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="15">
+    <tableColumn id="1" xr3:uid="{140526B3-4646-4B6D-ADF6-1795013DDCFE}" name="Scenario" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{FB458ACB-5E52-4905-8CA6-14F376434220}" name="What changes" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{FE9C9EDD-4FE5-47F7-B930-B7A16D0782BF}" name="Shift affiliate (EUR)" dataDxfId="12">
+      <calculatedColumnFormula>1.5</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{0508E6B3-7595-4F25-BE11-CE6CBBB48B0F}" name="Shift paid_search (EUR)" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{DCF123D4-D763-4BB9-83FA-568CC7A33727}" name="Shift paid_social (EUR)" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{2BE29272-FA4B-4096-82B5-7A75B59E7BD8}" name="Shift referral (EUR)" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{E469D44F-21D9-4497-928A-956A4947E1CC}" name="affiliate spend (EUR)" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{8E936B22-0B22-4F95-A0AD-B6A047CDDD77}" name="paid_search spend (EUR)" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{C379554C-A418-4778-B585-5E0A99257B02}" name="paid_social spend (EUR)" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{9686B15B-2978-41FE-B9F3-F49505F605E2}" name="referral spend (EUR)" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{F898B0E9-E0F7-40CD-94E3-17C1FDCBE073}" name="Total spend (EUR)" dataDxfId="4">
+      <calculatedColumnFormula>SUM(G5:J5)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="12" xr3:uid="{25C2165C-A6DB-4BE7-9EF2-263BBEF20FE8}" name="Customers won" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{7381C361-DF7C-40A6-AAA3-4A7014BF184B}" name="Net profit at recommended spend (EUR)" dataDxfId="2"/>
+    <tableColumn id="14" xr3:uid="{43D75303-A39E-4B2B-8332-1DB0D9DEEB50}" name="Net profit at baseline spend (EUR)" dataDxfId="1"/>
+    <tableColumn id="15" xr3:uid="{96C86429-40AF-4FE1-B7A0-7704D4DF24C2}" name="Uplift (EUR)" dataDxfId="0">
+      <calculatedColumnFormula>M5-N5</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -5644,70 +6299,70 @@
       </c>
     </row>
     <row r="21" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="60" t="s">
+      <c r="A21" s="84" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="59"/>
-      <c r="C21" s="59"/>
-      <c r="D21" s="59"/>
-      <c r="E21" s="59"/>
-      <c r="F21" s="59"/>
-      <c r="G21" s="59"/>
+      <c r="B21" s="83"/>
+      <c r="C21" s="83"/>
+      <c r="D21" s="83"/>
+      <c r="E21" s="83"/>
+      <c r="F21" s="83"/>
+      <c r="G21" s="83"/>
     </row>
     <row r="22" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="60" t="s">
+      <c r="A22" s="84" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="59"/>
-      <c r="C22" s="59"/>
-      <c r="D22" s="59"/>
-      <c r="E22" s="59"/>
-      <c r="F22" s="59"/>
-      <c r="G22" s="59"/>
+      <c r="B22" s="83"/>
+      <c r="C22" s="83"/>
+      <c r="D22" s="83"/>
+      <c r="E22" s="83"/>
+      <c r="F22" s="83"/>
+      <c r="G22" s="83"/>
     </row>
     <row r="23" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="60" t="s">
+      <c r="A23" s="84" t="s">
         <v>20</v>
       </c>
-      <c r="B23" s="59"/>
-      <c r="C23" s="59"/>
-      <c r="D23" s="59"/>
-      <c r="E23" s="59"/>
-      <c r="F23" s="59"/>
-      <c r="G23" s="59"/>
+      <c r="B23" s="83"/>
+      <c r="C23" s="83"/>
+      <c r="D23" s="83"/>
+      <c r="E23" s="83"/>
+      <c r="F23" s="83"/>
+      <c r="G23" s="83"/>
     </row>
     <row r="24" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="60" t="s">
+      <c r="A24" s="84" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="59"/>
-      <c r="C24" s="59"/>
-      <c r="D24" s="59"/>
-      <c r="E24" s="59"/>
-      <c r="F24" s="59"/>
-      <c r="G24" s="59"/>
+      <c r="B24" s="83"/>
+      <c r="C24" s="83"/>
+      <c r="D24" s="83"/>
+      <c r="E24" s="83"/>
+      <c r="F24" s="83"/>
+      <c r="G24" s="83"/>
     </row>
     <row r="25" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="60" t="s">
+      <c r="A25" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="59"/>
-      <c r="C25" s="59"/>
-      <c r="D25" s="59"/>
-      <c r="E25" s="59"/>
-      <c r="F25" s="59"/>
-      <c r="G25" s="59"/>
+      <c r="B25" s="83"/>
+      <c r="C25" s="83"/>
+      <c r="D25" s="83"/>
+      <c r="E25" s="83"/>
+      <c r="F25" s="83"/>
+      <c r="G25" s="83"/>
     </row>
     <row r="27" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="58" t="s">
+      <c r="A27" s="82" t="s">
         <v>23</v>
       </c>
-      <c r="B27" s="59"/>
-      <c r="C27" s="59"/>
-      <c r="D27" s="59"/>
-      <c r="E27" s="59"/>
-      <c r="F27" s="59"/>
-      <c r="G27" s="59"/>
+      <c r="B27" s="83"/>
+      <c r="C27" s="83"/>
+      <c r="D27" s="83"/>
+      <c r="E27" s="83"/>
+      <c r="F27" s="83"/>
+      <c r="G27" s="83"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
@@ -5753,6 +6408,1198 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D41B753-3D14-4CD8-A6D6-4EDEC0B396DF}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02FD9BB6-92B3-41DA-B0A3-8137671C795C}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C01AF9F-AE8A-4B2F-97D1-ABA6C3D76678}">
+  <dimension ref="A1:F50"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.77734375" style="48" customWidth="1"/>
+    <col min="2" max="7" width="12.77734375" style="48" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="48"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A1" s="51" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="50" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="56" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A5" s="52" t="s">
+        <v>224</v>
+      </c>
+      <c r="B5" s="52" t="s">
+        <v>215</v>
+      </c>
+      <c r="C5"/>
+      <c r="D5"/>
+      <c r="E5"/>
+      <c r="F5"/>
+    </row>
+    <row r="6" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="52" t="s">
+        <v>213</v>
+      </c>
+      <c r="B6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" t="s">
+        <v>69</v>
+      </c>
+      <c r="E6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F6" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="53" t="s">
+        <v>216</v>
+      </c>
+      <c r="B7" s="54">
+        <v>3700.24</v>
+      </c>
+      <c r="C7" s="54">
+        <v>5445.75</v>
+      </c>
+      <c r="D7" s="54">
+        <v>8042.77</v>
+      </c>
+      <c r="E7" s="54">
+        <v>1340.53</v>
+      </c>
+      <c r="F7" s="54">
+        <v>18529.29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A8" s="53" t="s">
+        <v>217</v>
+      </c>
+      <c r="B8" s="54">
+        <v>2219.08</v>
+      </c>
+      <c r="C8" s="54">
+        <v>4812.82</v>
+      </c>
+      <c r="D8" s="54">
+        <v>6017.4</v>
+      </c>
+      <c r="E8" s="54">
+        <v>979.58999999999992</v>
+      </c>
+      <c r="F8" s="54">
+        <v>14028.89</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="53" t="s">
+        <v>218</v>
+      </c>
+      <c r="B9" s="54">
+        <v>2419.5199999999995</v>
+      </c>
+      <c r="C9" s="54">
+        <v>5129.18</v>
+      </c>
+      <c r="D9" s="54">
+        <v>6144.2900000000009</v>
+      </c>
+      <c r="E9" s="54">
+        <v>946.43000000000006</v>
+      </c>
+      <c r="F9" s="54">
+        <v>14639.420000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A10" s="53" t="s">
+        <v>219</v>
+      </c>
+      <c r="B10" s="54">
+        <v>2452.1099999999997</v>
+      </c>
+      <c r="C10" s="54">
+        <v>4997</v>
+      </c>
+      <c r="D10" s="54">
+        <v>6065.59</v>
+      </c>
+      <c r="E10" s="54">
+        <v>1027.5700000000002</v>
+      </c>
+      <c r="F10" s="54">
+        <v>14542.27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A11" s="53" t="s">
+        <v>220</v>
+      </c>
+      <c r="B11" s="54">
+        <v>4148.6100000000006</v>
+      </c>
+      <c r="C11" s="54">
+        <v>7611.43</v>
+      </c>
+      <c r="D11" s="54">
+        <v>11317.44</v>
+      </c>
+      <c r="E11" s="54">
+        <v>1195.72</v>
+      </c>
+      <c r="F11" s="54">
+        <v>24273.200000000004</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="53" t="s">
+        <v>221</v>
+      </c>
+      <c r="B12" s="54">
+        <v>2849.87</v>
+      </c>
+      <c r="C12" s="54">
+        <v>6257.49</v>
+      </c>
+      <c r="D12" s="54">
+        <v>6411.41</v>
+      </c>
+      <c r="E12" s="54">
+        <v>988.06</v>
+      </c>
+      <c r="F12" s="54">
+        <v>16506.830000000002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A13" s="53" t="s">
+        <v>222</v>
+      </c>
+      <c r="B13" s="54">
+        <v>2771.6800000000003</v>
+      </c>
+      <c r="C13" s="54">
+        <v>6052.7400000000007</v>
+      </c>
+      <c r="D13" s="54">
+        <v>10944.369999999999</v>
+      </c>
+      <c r="E13" s="54">
+        <v>1159.55</v>
+      </c>
+      <c r="F13" s="54">
+        <v>20928.34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A14" s="53" t="s">
+        <v>223</v>
+      </c>
+      <c r="B14" s="54">
+        <v>3116.48</v>
+      </c>
+      <c r="C14" s="54">
+        <v>5374.79</v>
+      </c>
+      <c r="D14" s="54">
+        <v>19030.080000000002</v>
+      </c>
+      <c r="E14" s="54">
+        <v>1081.3399999999999</v>
+      </c>
+      <c r="F14" s="54">
+        <v>28602.690000000002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="53" t="s">
+        <v>214</v>
+      </c>
+      <c r="B15" s="54">
+        <v>23677.59</v>
+      </c>
+      <c r="C15" s="54">
+        <v>45681.2</v>
+      </c>
+      <c r="D15" s="54">
+        <v>73973.349999999991</v>
+      </c>
+      <c r="E15" s="54">
+        <v>8718.7900000000009</v>
+      </c>
+      <c r="F15" s="54">
+        <v>152050.93</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A16"/>
+      <c r="B16"/>
+      <c r="C16"/>
+    </row>
+    <row r="17" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A17"/>
+      <c r="B17"/>
+      <c r="C17"/>
+    </row>
+    <row r="18" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A18" s="57" t="s">
+        <v>135</v>
+      </c>
+      <c r="B18"/>
+      <c r="C18"/>
+    </row>
+    <row r="19" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A19" s="52" t="s">
+        <v>225</v>
+      </c>
+      <c r="B19" s="52" t="s">
+        <v>215</v>
+      </c>
+      <c r="C19"/>
+      <c r="D19"/>
+      <c r="E19"/>
+      <c r="F19"/>
+    </row>
+    <row r="20" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A20" s="52" t="s">
+        <v>213</v>
+      </c>
+      <c r="B20" t="s">
+        <v>62</v>
+      </c>
+      <c r="C20" t="s">
+        <v>67</v>
+      </c>
+      <c r="D20" t="s">
+        <v>69</v>
+      </c>
+      <c r="E20" t="s">
+        <v>71</v>
+      </c>
+      <c r="F20" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="53" t="s">
+        <v>216</v>
+      </c>
+      <c r="B21" s="54">
+        <v>97.3</v>
+      </c>
+      <c r="C21" s="54">
+        <v>230.52</v>
+      </c>
+      <c r="D21" s="54">
+        <v>115.52000000000001</v>
+      </c>
+      <c r="E21" s="54">
+        <v>111.77000000000001</v>
+      </c>
+      <c r="F21" s="54">
+        <v>555.11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A22" s="53" t="s">
+        <v>217</v>
+      </c>
+      <c r="B22" s="54">
+        <v>96.259999999999991</v>
+      </c>
+      <c r="C22" s="54">
+        <v>211.82</v>
+      </c>
+      <c r="D22" s="54">
+        <v>95.66</v>
+      </c>
+      <c r="E22" s="54">
+        <v>116.5</v>
+      </c>
+      <c r="F22" s="54">
+        <v>520.24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A23" s="53" t="s">
+        <v>218</v>
+      </c>
+      <c r="B23" s="54">
+        <v>90.740000000000009</v>
+      </c>
+      <c r="C23" s="54">
+        <v>227.65</v>
+      </c>
+      <c r="D23" s="54">
+        <v>113.56</v>
+      </c>
+      <c r="E23" s="54">
+        <v>98.47</v>
+      </c>
+      <c r="F23" s="54">
+        <v>530.41999999999996</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A24" s="53" t="s">
+        <v>219</v>
+      </c>
+      <c r="B24" s="54">
+        <v>85.22999999999999</v>
+      </c>
+      <c r="C24" s="54">
+        <v>202.23000000000002</v>
+      </c>
+      <c r="D24" s="54">
+        <v>129.5</v>
+      </c>
+      <c r="E24" s="54">
+        <v>104.87</v>
+      </c>
+      <c r="F24" s="54">
+        <v>521.83000000000004</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A25" s="53" t="s">
+        <v>220</v>
+      </c>
+      <c r="B25" s="54">
+        <v>140.46</v>
+      </c>
+      <c r="C25" s="54">
+        <v>268.7</v>
+      </c>
+      <c r="D25" s="54">
+        <v>159.36000000000001</v>
+      </c>
+      <c r="E25" s="54">
+        <v>109.36999999999999</v>
+      </c>
+      <c r="F25" s="54">
+        <v>677.89</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A26" s="53" t="s">
+        <v>221</v>
+      </c>
+      <c r="B26" s="54">
+        <v>109.84</v>
+      </c>
+      <c r="C26" s="54">
+        <v>267.16000000000003</v>
+      </c>
+      <c r="D26" s="54">
+        <v>126.93</v>
+      </c>
+      <c r="E26" s="54">
+        <v>100.7</v>
+      </c>
+      <c r="F26" s="54">
+        <v>604.63</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A27" s="53" t="s">
+        <v>222</v>
+      </c>
+      <c r="B27" s="54">
+        <v>113.63</v>
+      </c>
+      <c r="C27" s="54">
+        <v>261.97000000000003</v>
+      </c>
+      <c r="D27" s="54">
+        <v>120.43</v>
+      </c>
+      <c r="E27" s="54">
+        <v>111.67</v>
+      </c>
+      <c r="F27" s="54">
+        <v>607.70000000000005</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A28" s="53" t="s">
+        <v>223</v>
+      </c>
+      <c r="B28" s="54">
+        <v>115.53999999999999</v>
+      </c>
+      <c r="C28" s="54">
+        <v>222.13</v>
+      </c>
+      <c r="D28" s="54">
+        <v>120.43</v>
+      </c>
+      <c r="E28" s="54">
+        <v>109.13999999999999</v>
+      </c>
+      <c r="F28" s="54">
+        <v>567.24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A29" s="53" t="s">
+        <v>214</v>
+      </c>
+      <c r="B29" s="54">
+        <v>849</v>
+      </c>
+      <c r="C29" s="54">
+        <v>1892.1800000000003</v>
+      </c>
+      <c r="D29" s="54">
+        <v>981.3900000000001</v>
+      </c>
+      <c r="E29" s="54">
+        <v>862.49</v>
+      </c>
+      <c r="F29" s="54">
+        <v>4585.0599999999995</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A30"/>
+      <c r="B30"/>
+      <c r="C30"/>
+    </row>
+    <row r="31" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A31"/>
+      <c r="B31"/>
+      <c r="C31"/>
+    </row>
+    <row r="32" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A32" s="57" t="s">
+        <v>226</v>
+      </c>
+      <c r="B32"/>
+      <c r="C32"/>
+    </row>
+    <row r="33" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A33" s="52" t="s">
+        <v>227</v>
+      </c>
+      <c r="B33" s="52" t="s">
+        <v>215</v>
+      </c>
+      <c r="C33"/>
+      <c r="D33"/>
+      <c r="E33"/>
+      <c r="F33"/>
+    </row>
+    <row r="34" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A34" s="52" t="s">
+        <v>213</v>
+      </c>
+      <c r="B34" t="s">
+        <v>62</v>
+      </c>
+      <c r="C34" t="s">
+        <v>67</v>
+      </c>
+      <c r="D34" t="s">
+        <v>69</v>
+      </c>
+      <c r="E34" t="s">
+        <v>71</v>
+      </c>
+      <c r="F34" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A35" s="53" t="s">
+        <v>216</v>
+      </c>
+      <c r="B35" s="55">
+        <v>38.029188078108938</v>
+      </c>
+      <c r="C35" s="55">
+        <v>23.623763664757938</v>
+      </c>
+      <c r="D35" s="55">
+        <v>69.62231648199446</v>
+      </c>
+      <c r="E35" s="55">
+        <v>11.993647669320925</v>
+      </c>
+      <c r="F35" s="55">
+        <v>33.379492352866997</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A36" s="53" t="s">
+        <v>217</v>
+      </c>
+      <c r="B36" s="55">
+        <v>23.05298150841471</v>
+      </c>
+      <c r="C36" s="55">
+        <v>22.721272778774431</v>
+      </c>
+      <c r="D36" s="55">
+        <v>62.904035124398909</v>
+      </c>
+      <c r="E36" s="55">
+        <v>8.4084978540772521</v>
+      </c>
+      <c r="F36" s="55">
+        <v>26.966188682146701</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A37" s="53" t="s">
+        <v>218</v>
+      </c>
+      <c r="B37" s="55">
+        <v>26.664315627066337</v>
+      </c>
+      <c r="C37" s="55">
+        <v>22.530990555677576</v>
+      </c>
+      <c r="D37" s="55">
+        <v>54.106111306798176</v>
+      </c>
+      <c r="E37" s="55">
+        <v>9.6113537117903931</v>
+      </c>
+      <c r="F37" s="55">
+        <v>27.599675728667844</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A38" s="53" t="s">
+        <v>219</v>
+      </c>
+      <c r="B38" s="55">
+        <v>28.770503343892994</v>
+      </c>
+      <c r="C38" s="55">
+        <v>24.709489195470503</v>
+      </c>
+      <c r="D38" s="55">
+        <v>46.838532818532819</v>
+      </c>
+      <c r="E38" s="55">
+        <v>9.7985124439782592</v>
+      </c>
+      <c r="F38" s="55">
+        <v>27.867830519517845</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A39" s="53" t="s">
+        <v>220</v>
+      </c>
+      <c r="B39" s="55">
+        <v>29.535882101665958</v>
+      </c>
+      <c r="C39" s="55">
+        <v>28.326870115370305</v>
+      </c>
+      <c r="D39" s="55">
+        <v>71.018072289156621</v>
+      </c>
+      <c r="E39" s="55">
+        <v>10.932796927859561</v>
+      </c>
+      <c r="F39" s="55">
+        <v>35.80698933455281</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A40" s="53" t="s">
+        <v>221</v>
+      </c>
+      <c r="B40" s="55">
+        <v>25.945648215586306</v>
+      </c>
+      <c r="C40" s="55">
+        <v>23.422256325797271</v>
+      </c>
+      <c r="D40" s="55">
+        <v>50.511384227526982</v>
+      </c>
+      <c r="E40" s="55">
+        <v>9.8119165839126108</v>
+      </c>
+      <c r="F40" s="55">
+        <v>27.300712832641441</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A41" s="53" t="s">
+        <v>222</v>
+      </c>
+      <c r="B41" s="55">
+        <v>24.392149960397784</v>
+      </c>
+      <c r="C41" s="55">
+        <v>23.104706645799137</v>
+      </c>
+      <c r="D41" s="55">
+        <v>90.877439176284966</v>
+      </c>
+      <c r="E41" s="55">
+        <v>10.383719888958538</v>
+      </c>
+      <c r="F41" s="55">
+        <v>34.438604574625636</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A42" s="53" t="s">
+        <v>223</v>
+      </c>
+      <c r="B42" s="55">
+        <v>26.973169465120307</v>
+      </c>
+      <c r="C42" s="55">
+        <v>24.196596587583848</v>
+      </c>
+      <c r="D42" s="55">
+        <v>158.01776965872293</v>
+      </c>
+      <c r="E42" s="55">
+        <v>9.907824812167858</v>
+      </c>
+      <c r="F42" s="55">
+        <v>50.424317749100915</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A43" s="53" t="s">
+        <v>214</v>
+      </c>
+      <c r="B43" s="55">
+        <v>27.888798586572442</v>
+      </c>
+      <c r="C43" s="55">
+        <v>24.142100645815944</v>
+      </c>
+      <c r="D43" s="55">
+        <v>75.376099206227906</v>
+      </c>
+      <c r="E43" s="55">
+        <v>10.108859233150529</v>
+      </c>
+      <c r="F43" s="55">
+        <v>33.162255237663196</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A44"/>
+      <c r="B44"/>
+      <c r="C44"/>
+    </row>
+    <row r="45" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A45"/>
+      <c r="B45"/>
+      <c r="C45"/>
+    </row>
+    <row r="46" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A46"/>
+      <c r="B46"/>
+      <c r="C46"/>
+    </row>
+    <row r="47" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A47"/>
+      <c r="B47"/>
+      <c r="C47"/>
+    </row>
+    <row r="48" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A48"/>
+      <c r="B48"/>
+      <c r="C48"/>
+    </row>
+    <row r="49" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A49"/>
+      <c r="B49"/>
+      <c r="C49"/>
+    </row>
+    <row r="50" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A50"/>
+      <c r="B50"/>
+      <c r="C50"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId4"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="120" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="41" t="s">
+        <v>157</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="41" t="s">
+        <v>159</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="41" t="s">
+        <v>163</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="41" t="s">
+        <v>165</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="41" t="s">
+        <v>167</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="41" t="s">
+        <v>168</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="41" t="s">
+        <v>170</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="41" t="s">
+        <v>172</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="46" t="s">
+        <v>205</v>
+      </c>
+      <c r="B13" s="47" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="B14" s="47" t="s">
+        <v>208</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:Q9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="17" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="P1" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="Q1" s="5" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A2" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" s="15">
+        <v>23677.59</v>
+      </c>
+      <c r="C2" s="15">
+        <v>846</v>
+      </c>
+      <c r="D2" s="15">
+        <v>1368</v>
+      </c>
+      <c r="E2" s="15">
+        <v>3420</v>
+      </c>
+      <c r="F2" s="15">
+        <v>32.03</v>
+      </c>
+      <c r="G2" s="15">
+        <v>27.99</v>
+      </c>
+      <c r="H2" s="15">
+        <v>382</v>
+      </c>
+      <c r="I2" s="15">
+        <v>251.54</v>
+      </c>
+      <c r="J2" s="15">
+        <v>321.20999999999998</v>
+      </c>
+      <c r="K2" s="15">
+        <v>7.8529999999999998</v>
+      </c>
+      <c r="L2" s="15">
+        <v>11.477</v>
+      </c>
+      <c r="M2" s="15">
+        <v>3</v>
+      </c>
+      <c r="N2" s="15">
+        <v>1</v>
+      </c>
+      <c r="O2" s="15">
+        <v>742.49</v>
+      </c>
+      <c r="P2" s="15">
+        <v>-490.95</v>
+      </c>
+      <c r="Q2" s="15">
+        <v>-15.327999999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A3" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" s="15">
+        <v>0</v>
+      </c>
+      <c r="C3" s="15">
+        <v>1401</v>
+      </c>
+      <c r="D3" s="15">
+        <v>1831</v>
+      </c>
+      <c r="E3" s="15">
+        <v>4577.5</v>
+      </c>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15">
+        <v>650</v>
+      </c>
+      <c r="I3" s="15">
+        <v>167.97</v>
+      </c>
+      <c r="J3" s="15">
+        <v>217.02</v>
+      </c>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="15"/>
+      <c r="N3" s="15"/>
+      <c r="O3" s="15">
+        <v>196.21</v>
+      </c>
+      <c r="P3" s="15">
+        <v>-28.24</v>
+      </c>
+      <c r="Q3" s="15"/>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A4" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" s="15">
+        <v>45681.2</v>
+      </c>
+      <c r="C4" s="15">
+        <v>1545</v>
+      </c>
+      <c r="D4" s="15">
+        <v>2086</v>
+      </c>
+      <c r="E4" s="15">
+        <v>5215</v>
+      </c>
+      <c r="F4" s="15">
+        <v>32.94</v>
+      </c>
+      <c r="G4" s="15">
+        <v>29.57</v>
+      </c>
+      <c r="H4" s="15">
+        <v>719</v>
+      </c>
+      <c r="I4" s="15">
+        <v>185.36</v>
+      </c>
+      <c r="J4" s="15">
+        <v>237.31</v>
+      </c>
+      <c r="K4" s="15">
+        <v>5.6269999999999998</v>
+      </c>
+      <c r="L4" s="15">
+        <v>8.0259999999999998</v>
+      </c>
+      <c r="M4" s="15">
+        <v>4</v>
+      </c>
+      <c r="N4" s="15">
+        <v>1</v>
+      </c>
+      <c r="O4" s="15">
+        <v>217.32</v>
+      </c>
+      <c r="P4" s="15">
+        <v>-31.96</v>
+      </c>
+      <c r="Q4" s="15">
+        <v>-0.97</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A5" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="B5" s="15">
+        <v>73973.350000000006</v>
+      </c>
+      <c r="C5" s="15">
+        <v>1225</v>
+      </c>
+      <c r="D5" s="15">
+        <v>2550</v>
+      </c>
+      <c r="E5" s="15">
+        <v>6375</v>
+      </c>
+      <c r="F5" s="15">
+        <v>65.59</v>
+      </c>
+      <c r="G5" s="15">
+        <v>60.39</v>
+      </c>
+      <c r="H5" s="15">
+        <v>562</v>
+      </c>
+      <c r="I5" s="15">
+        <v>171.28</v>
+      </c>
+      <c r="J5" s="15">
+        <v>216.32</v>
+      </c>
+      <c r="K5" s="15">
+        <v>2.6110000000000002</v>
+      </c>
+      <c r="L5" s="15">
+        <v>3.5819999999999999</v>
+      </c>
+      <c r="M5" s="15">
+        <v>6</v>
+      </c>
+      <c r="N5" s="15">
+        <v>1</v>
+      </c>
+      <c r="O5" s="15">
+        <v>225.31</v>
+      </c>
+      <c r="P5" s="15">
+        <v>-54.03</v>
+      </c>
+      <c r="Q5" s="15">
+        <v>-0.82399999999999995</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A6" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="15">
+        <v>8718.7900000000009</v>
+      </c>
+      <c r="C6" s="15">
+        <v>911</v>
+      </c>
+      <c r="D6" s="15">
+        <v>1056</v>
+      </c>
+      <c r="E6" s="15">
+        <v>2640</v>
+      </c>
+      <c r="F6" s="15">
+        <v>12.47</v>
+      </c>
+      <c r="G6" s="15">
+        <v>9.57</v>
+      </c>
+      <c r="H6" s="15">
+        <v>467</v>
+      </c>
+      <c r="I6" s="15">
+        <v>165.36</v>
+      </c>
+      <c r="J6" s="15">
+        <v>217.06</v>
+      </c>
+      <c r="K6" s="15">
+        <v>13.262</v>
+      </c>
+      <c r="L6" s="15">
+        <v>22.68</v>
+      </c>
+      <c r="M6" s="15">
+        <v>2</v>
+      </c>
+      <c r="N6" s="15">
+        <v>1</v>
+      </c>
+      <c r="O6" s="15">
+        <v>110.87</v>
+      </c>
+      <c r="P6" s="15">
+        <v>54.49</v>
+      </c>
+      <c r="Q6" s="15">
+        <v>4.3710000000000004</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:J97"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -8584,7 +10431,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:G61"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -9642,7 +11489,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -9890,16 +11737,114 @@
       </c>
     </row>
     <row r="23" spans="1:4" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="58" t="s">
+      <c r="A23" s="82" t="s">
         <v>73</v>
       </c>
-      <c r="B23" s="59"/>
-      <c r="C23" s="59"/>
-      <c r="D23" s="59"/>
+      <c r="B23" s="83"/>
+      <c r="C23" s="83"/>
+      <c r="D23" s="83"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A26" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="B27" s="20">
+        <v>0</v>
+      </c>
+      <c r="C27" s="45">
+        <v>-220.92</v>
+      </c>
+      <c r="D27" s="76">
+        <v>206.55</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="B28" s="20">
+        <v>0</v>
+      </c>
+      <c r="C28" s="45">
+        <v>-98.22</v>
+      </c>
+      <c r="D28" s="76">
+        <v>83.53</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="B29" s="20">
+        <v>0</v>
+      </c>
+      <c r="C29" s="45">
+        <v>-87.43</v>
+      </c>
+      <c r="D29" s="76">
+        <v>78.400000000000006</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="B30" s="20">
+        <v>0</v>
+      </c>
+      <c r="C30" s="45">
+        <v>-87.67</v>
+      </c>
+      <c r="D30" s="76">
+        <v>83.55</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="B31" s="20">
+        <v>0</v>
+      </c>
+      <c r="C31" s="45">
+        <v>-98.15</v>
+      </c>
+      <c r="D31" s="76">
+        <v>76.150000000000006</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="86" t="s">
+        <v>232</v>
+      </c>
+      <c r="B32" s="85"/>
+      <c r="C32" s="85"/>
+      <c r="D32" s="85"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A32:D32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10063,7 +12008,7 @@
         <v>0</v>
       </c>
       <c r="Q5" s="32">
-        <f>J5+P5-O5</f>
+        <f>J5+P5-O5+Assumptions!B27</f>
         <v>-490.95000000000005</v>
       </c>
       <c r="R5" s="31">
@@ -10145,7 +12090,7 @@
         <v>0</v>
       </c>
       <c r="Q6" s="32">
-        <f>J6+P6-O6</f>
+        <f>J6+P6-O6+Assumptions!B28</f>
         <v>-28.240000000000009</v>
       </c>
       <c r="R6" s="31" t="str">
@@ -10227,7 +12172,7 @@
         <v>0</v>
       </c>
       <c r="Q7" s="32">
-        <f>J7+P7-O7</f>
+        <f>J7+P7-O7+Assumptions!B29</f>
         <v>-31.95999999999998</v>
       </c>
       <c r="R7" s="31">
@@ -10309,7 +12254,7 @@
         <v>0</v>
       </c>
       <c r="Q8" s="32">
-        <f>J8+P8-O8</f>
+        <f>J8+P8-O8+Assumptions!B30</f>
         <v>-54.03</v>
       </c>
       <c r="R8" s="31">
@@ -10391,7 +12336,7 @@
         <v>0</v>
       </c>
       <c r="Q9" s="32">
-        <f>J9+P9-O9</f>
+        <f>J9+P9-O9+Assumptions!B31</f>
         <v>54.490000000000009</v>
       </c>
       <c r="R9" s="31">
@@ -10958,18 +12903,18 @@
       </c>
     </row>
     <row r="10" spans="1:10" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="58" t="s">
+      <c r="A10" s="82" t="s">
         <v>106</v>
       </c>
-      <c r="B10" s="59"/>
-      <c r="C10" s="59"/>
-      <c r="D10" s="59"/>
-      <c r="E10" s="59"/>
-      <c r="F10" s="59"/>
-      <c r="G10" s="59"/>
-      <c r="H10" s="59"/>
-      <c r="I10" s="59"/>
-      <c r="J10" s="59"/>
+      <c r="B10" s="83"/>
+      <c r="C10" s="83"/>
+      <c r="D10" s="83"/>
+      <c r="E10" s="83"/>
+      <c r="F10" s="83"/>
+      <c r="G10" s="83"/>
+      <c r="H10" s="83"/>
+      <c r="I10" s="83"/>
+      <c r="J10" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11008,42 +12953,42 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="60" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="64" t="s">
+      <c r="B4" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="C4" s="64" t="s">
+      <c r="C4" s="61" t="s">
         <v>110</v>
       </c>
-      <c r="D4" s="64" t="s">
+      <c r="D4" s="61" t="s">
         <v>111</v>
       </c>
-      <c r="E4" s="64" t="s">
+      <c r="E4" s="61" t="s">
         <v>112</v>
       </c>
-      <c r="F4" s="64" t="s">
+      <c r="F4" s="61" t="s">
         <v>113</v>
       </c>
-      <c r="G4" s="64" t="s">
+      <c r="G4" s="61" t="s">
         <v>114</v>
       </c>
-      <c r="H4" s="64" t="s">
+      <c r="H4" s="61" t="s">
         <v>115</v>
       </c>
-      <c r="I4" s="64" t="s">
+      <c r="I4" s="61" t="s">
         <v>93</v>
       </c>
-      <c r="J4" s="64" t="s">
+      <c r="J4" s="61" t="s">
         <v>116</v>
       </c>
-      <c r="K4" s="65" t="s">
+      <c r="K4" s="62" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="61" t="s">
+      <c r="A5" s="58" t="s">
         <v>62</v>
       </c>
       <c r="B5" s="10">
@@ -11081,13 +13026,13 @@
         <f>G5*I5</f>
         <v>-53308.848979121671</v>
       </c>
-      <c r="K5" s="62">
+      <c r="K5" s="59">
         <f>H5*I5</f>
         <v>-34191.304622922937</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="61" t="s">
+      <c r="A6" s="58" t="s">
         <v>67</v>
       </c>
       <c r="B6" s="10">
@@ -11125,13 +13070,13 @@
         <f>G6*I6</f>
         <v>-8025.8318512750729</v>
       </c>
-      <c r="K6" s="62">
+      <c r="K6" s="59">
         <f>H6*I6</f>
         <v>-4970.2238896687222</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="61" t="s">
+      <c r="A7" s="58" t="s">
         <v>69</v>
       </c>
       <c r="B7" s="10">
@@ -11169,51 +13114,51 @@
         <f>G7*I7</f>
         <v>-13152.044318661221</v>
       </c>
-      <c r="K7" s="62">
+      <c r="K7" s="59">
         <f>H7*I7</f>
         <v>-8579.6142933444535</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="66" t="s">
+      <c r="A8" s="63" t="s">
         <v>71</v>
       </c>
-      <c r="B8" s="67">
+      <c r="B8" s="64">
         <f>SUMIFS(Data_Monthly!$C$2:$C$97,Data_Monthly!$A$2:$A$97,A8,Data_Monthly!$E$2:$E$97,1)</f>
         <v>1081.3399999999999</v>
       </c>
-      <c r="C8" s="67">
+      <c r="C8" s="64">
         <f>B8*Assumptions!$B$9</f>
         <v>540.66999999999996</v>
       </c>
-      <c r="D8" s="67">
+      <c r="D8" s="64">
         <f>B8*IF(A8="referral",Assumptions!$B$11,Assumptions!$B$10)</f>
         <v>1297.6079999999999</v>
       </c>
-      <c r="E8" s="68">
+      <c r="E8" s="65">
         <v>1297.6079999999999</v>
       </c>
-      <c r="F8" s="69">
+      <c r="F8" s="66">
         <f>E8/B8-1</f>
         <v>0.19999999999999996</v>
       </c>
-      <c r="G8" s="70">
+      <c r="G8" s="67">
         <f>Assumptions!$B$6*Curves!E8*(B8/Assumptions!$B$6)^Curves!C8</f>
         <v>107.10507367059948</v>
       </c>
-      <c r="H8" s="70">
+      <c r="H8" s="67">
         <f>Assumptions!$B$6*Curves!E8*(E8/Assumptions!$B$6)^Curves!C8</f>
         <v>115.44823882568373</v>
       </c>
-      <c r="I8" s="71">
+      <c r="I8" s="68">
         <f>VLOOKUP(A8,Unit_Economics!$A$5:$T$9,20,FALSE)</f>
         <v>51.592085620197594</v>
       </c>
-      <c r="J8" s="67">
+      <c r="J8" s="64">
         <f>G8*I8</f>
         <v>5525.7741311711397</v>
       </c>
-      <c r="K8" s="72">
+      <c r="K8" s="69">
         <f>H8*I8</f>
         <v>5956.2154221956953</v>
       </c>
@@ -11318,19 +13263,19 @@
       </c>
     </row>
     <row r="19" spans="1:11" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="58" t="s">
+      <c r="A19" s="82" t="s">
         <v>125</v>
       </c>
-      <c r="B19" s="59"/>
-      <c r="C19" s="59"/>
-      <c r="D19" s="59"/>
-      <c r="E19" s="59"/>
-      <c r="F19" s="59"/>
-      <c r="G19" s="59"/>
-      <c r="H19" s="59"/>
-      <c r="I19" s="59"/>
-      <c r="J19" s="59"/>
-      <c r="K19" s="59"/>
+      <c r="B19" s="83"/>
+      <c r="C19" s="83"/>
+      <c r="D19" s="83"/>
+      <c r="E19" s="83"/>
+      <c r="F19" s="83"/>
+      <c r="G19" s="83"/>
+      <c r="H19" s="83"/>
+      <c r="I19" s="83"/>
+      <c r="J19" s="83"/>
+      <c r="K19" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11374,45 +13319,45 @@
       </c>
     </row>
     <row r="4" spans="1:12" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="B4" s="64" t="s">
+      <c r="B4" s="61" t="s">
         <v>129</v>
       </c>
-      <c r="C4" s="64" t="s">
+      <c r="C4" s="61" t="s">
         <v>118</v>
       </c>
-      <c r="D4" s="64" t="s">
+      <c r="D4" s="61" t="s">
         <v>130</v>
       </c>
-      <c r="E4" s="64" t="s">
+      <c r="E4" s="61" t="s">
         <v>131</v>
       </c>
-      <c r="F4" s="64" t="s">
+      <c r="F4" s="61" t="s">
         <v>132</v>
       </c>
-      <c r="G4" s="64" t="s">
+      <c r="G4" s="61" t="s">
         <v>133</v>
       </c>
-      <c r="H4" s="64" t="s">
+      <c r="H4" s="61" t="s">
         <v>134</v>
       </c>
-      <c r="I4" s="64" t="s">
+      <c r="I4" s="61" t="s">
         <v>135</v>
       </c>
-      <c r="J4" s="64" t="s">
+      <c r="J4" s="61" t="s">
         <v>136</v>
       </c>
-      <c r="K4" s="64" t="s">
+      <c r="K4" s="61" t="s">
         <v>120</v>
       </c>
-      <c r="L4" s="65" t="s">
+      <c r="L4" s="62" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="73" t="s">
+      <c r="A5" s="70" t="s">
         <v>138</v>
       </c>
       <c r="B5" s="19" t="s">
@@ -11446,13 +13391,13 @@
       <c r="K5" s="10">
         <v>-97563.64</v>
       </c>
-      <c r="L5" s="74">
+      <c r="L5" s="71">
         <f t="shared" ref="L5:L12" si="1">J5-K5</f>
         <v>40720.43</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="73" t="s">
+      <c r="A6" s="70" t="s">
         <v>140</v>
       </c>
       <c r="B6" s="19" t="s">
@@ -11486,13 +13431,13 @@
       <c r="K6" s="10">
         <v>-97563.64</v>
       </c>
-      <c r="L6" s="74">
+      <c r="L6" s="71">
         <f t="shared" si="1"/>
         <v>40720.43</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="73" t="s">
+      <c r="A7" s="70" t="s">
         <v>142</v>
       </c>
       <c r="B7" s="19" t="s">
@@ -11526,13 +13471,13 @@
       <c r="K7" s="10">
         <v>-97563.64</v>
       </c>
-      <c r="L7" s="74">
+      <c r="L7" s="71">
         <f t="shared" si="1"/>
         <v>40720.43</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="73" t="s">
+      <c r="A8" s="70" t="s">
         <v>144</v>
       </c>
       <c r="B8" s="19" t="s">
@@ -11566,13 +13511,13 @@
       <c r="K8" s="10">
         <v>-145369.99</v>
       </c>
-      <c r="L8" s="74">
+      <c r="L8" s="71">
         <f t="shared" si="1"/>
         <v>56722.249999999985</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="73" t="s">
+      <c r="A9" s="70" t="s">
         <v>146</v>
       </c>
       <c r="B9" s="19" t="s">
@@ -11606,13 +13551,13 @@
       <c r="K9" s="10">
         <v>-49757.3</v>
       </c>
-      <c r="L9" s="74">
+      <c r="L9" s="71">
         <f t="shared" si="1"/>
         <v>24736.380000000005</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="73" t="s">
+      <c r="A10" s="70" t="s">
         <v>148</v>
       </c>
       <c r="B10" s="19" t="s">
@@ -11646,13 +13591,13 @@
       <c r="K10" s="10">
         <v>-92832.03</v>
       </c>
-      <c r="L10" s="74">
+      <c r="L10" s="71">
         <f t="shared" si="1"/>
         <v>37317.729999999996</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="73" t="s">
+      <c r="A11" s="70" t="s">
         <v>150</v>
       </c>
       <c r="B11" s="19" t="s">
@@ -11686,47 +13631,47 @@
       <c r="K11" s="10">
         <v>-62702.22</v>
       </c>
-      <c r="L11" s="74">
+      <c r="L11" s="71">
         <f t="shared" si="1"/>
         <v>30107.030000000002</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="75" t="s">
+      <c r="A12" s="72" t="s">
         <v>152</v>
       </c>
-      <c r="B12" s="76" t="s">
+      <c r="B12" s="73" t="s">
         <v>153</v>
       </c>
-      <c r="C12" s="67">
+      <c r="C12" s="64">
         <v>28603</v>
       </c>
-      <c r="D12" s="67">
+      <c r="D12" s="64">
         <v>1558</v>
       </c>
-      <c r="E12" s="67">
+      <c r="E12" s="64">
         <v>2687</v>
       </c>
-      <c r="F12" s="67">
+      <c r="F12" s="64">
         <v>22564</v>
       </c>
-      <c r="G12" s="67">
+      <c r="G12" s="64">
         <v>1298</v>
       </c>
-      <c r="H12" s="67">
+      <c r="H12" s="64">
         <f t="shared" si="0"/>
         <v>28107</v>
       </c>
-      <c r="I12" s="77">
+      <c r="I12" s="74">
         <v>572</v>
       </c>
-      <c r="J12" s="67">
+      <c r="J12" s="64">
         <v>-75920.679999999993</v>
       </c>
-      <c r="K12" s="67">
+      <c r="K12" s="64">
         <v>-97563.64</v>
       </c>
-      <c r="L12" s="78">
+      <c r="L12" s="75">
         <f t="shared" si="1"/>
         <v>21642.960000000006</v>
       </c>
@@ -11737,20 +13682,20 @@
       </c>
     </row>
     <row r="15" spans="1:12" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="58" t="s">
+      <c r="A15" s="82" t="s">
         <v>202</v>
       </c>
-      <c r="B15" s="59"/>
-      <c r="C15" s="59"/>
-      <c r="D15" s="59"/>
-      <c r="E15" s="59"/>
-      <c r="F15" s="59"/>
-      <c r="G15" s="59"/>
-      <c r="H15" s="59"/>
-      <c r="I15" s="59"/>
-      <c r="J15" s="59"/>
-      <c r="K15" s="59"/>
-      <c r="L15" s="59"/>
+      <c r="B15" s="83"/>
+      <c r="C15" s="83"/>
+      <c r="D15" s="83"/>
+      <c r="E15" s="83"/>
+      <c r="F15" s="83"/>
+      <c r="G15" s="83"/>
+      <c r="H15" s="83"/>
+      <c r="I15" s="83"/>
+      <c r="J15" s="83"/>
+      <c r="K15" s="83"/>
+      <c r="L15" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11764,1175 +13709,361 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C01AF9F-AE8A-4B2F-97D1-ABA6C3D76678}">
-  <dimension ref="A1:F50"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FAC0AE0-D9D8-460B-AA0B-BA9F0FFE1AA5}">
+  <dimension ref="A1:O11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.77734375" style="48" customWidth="1"/>
-    <col min="2" max="7" width="12.77734375" style="48" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="48"/>
+    <col min="1" max="1" width="30.77734375" customWidth="1"/>
+    <col min="2" max="2" width="52.77734375" customWidth="1"/>
+    <col min="3" max="15" width="16.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="51" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="50" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="56" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="52" t="s">
-        <v>224</v>
-      </c>
-      <c r="B5" s="52" t="s">
-        <v>215</v>
-      </c>
-      <c r="C5"/>
-      <c r="D5"/>
-      <c r="E5"/>
-      <c r="F5"/>
-    </row>
-    <row r="6" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="52" t="s">
-        <v>213</v>
-      </c>
-      <c r="B6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C6" t="s">
-        <v>67</v>
-      </c>
-      <c r="D6" t="s">
-        <v>69</v>
-      </c>
-      <c r="E6" t="s">
-        <v>71</v>
-      </c>
-      <c r="F6" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="53" t="s">
-        <v>216</v>
-      </c>
-      <c r="B7" s="54">
-        <v>3700.24</v>
-      </c>
-      <c r="C7" s="54">
-        <v>5445.75</v>
-      </c>
-      <c r="D7" s="54">
-        <v>8042.77</v>
-      </c>
-      <c r="E7" s="54">
-        <v>1340.53</v>
-      </c>
-      <c r="F7" s="54">
-        <v>18529.29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="53" t="s">
-        <v>217</v>
-      </c>
-      <c r="B8" s="54">
-        <v>2219.08</v>
-      </c>
-      <c r="C8" s="54">
-        <v>4812.82</v>
-      </c>
-      <c r="D8" s="54">
-        <v>6017.4</v>
-      </c>
-      <c r="E8" s="54">
-        <v>979.58999999999992</v>
-      </c>
-      <c r="F8" s="54">
-        <v>14028.89</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="53" t="s">
-        <v>218</v>
-      </c>
-      <c r="B9" s="54">
-        <v>2419.5199999999995</v>
-      </c>
-      <c r="C9" s="54">
-        <v>5129.18</v>
-      </c>
-      <c r="D9" s="54">
-        <v>6144.2900000000009</v>
-      </c>
-      <c r="E9" s="54">
-        <v>946.43000000000006</v>
-      </c>
-      <c r="F9" s="54">
-        <v>14639.420000000002</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="53" t="s">
-        <v>219</v>
-      </c>
-      <c r="B10" s="54">
-        <v>2452.1099999999997</v>
-      </c>
-      <c r="C10" s="54">
-        <v>4997</v>
-      </c>
-      <c r="D10" s="54">
-        <v>6065.59</v>
-      </c>
-      <c r="E10" s="54">
-        <v>1027.5700000000002</v>
-      </c>
-      <c r="F10" s="54">
-        <v>14542.27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A11" s="53" t="s">
-        <v>220</v>
-      </c>
-      <c r="B11" s="54">
-        <v>4148.6100000000006</v>
-      </c>
-      <c r="C11" s="54">
-        <v>7611.43</v>
-      </c>
-      <c r="D11" s="54">
-        <v>11317.44</v>
-      </c>
-      <c r="E11" s="54">
-        <v>1195.72</v>
-      </c>
-      <c r="F11" s="54">
-        <v>24273.200000000004</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="53" t="s">
-        <v>221</v>
-      </c>
-      <c r="B12" s="54">
-        <v>2849.87</v>
-      </c>
-      <c r="C12" s="54">
-        <v>6257.49</v>
-      </c>
-      <c r="D12" s="54">
-        <v>6411.41</v>
-      </c>
-      <c r="E12" s="54">
-        <v>988.06</v>
-      </c>
-      <c r="F12" s="54">
-        <v>16506.830000000002</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="53" t="s">
-        <v>222</v>
-      </c>
-      <c r="B13" s="54">
-        <v>2771.6800000000003</v>
-      </c>
-      <c r="C13" s="54">
-        <v>6052.7400000000007</v>
-      </c>
-      <c r="D13" s="54">
-        <v>10944.369999999999</v>
-      </c>
-      <c r="E13" s="54">
-        <v>1159.55</v>
-      </c>
-      <c r="F13" s="54">
-        <v>20928.34</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="53" t="s">
-        <v>223</v>
-      </c>
-      <c r="B14" s="54">
-        <v>3116.48</v>
-      </c>
-      <c r="C14" s="54">
-        <v>5374.79</v>
-      </c>
-      <c r="D14" s="54">
-        <v>19030.080000000002</v>
-      </c>
-      <c r="E14" s="54">
-        <v>1081.3399999999999</v>
-      </c>
-      <c r="F14" s="54">
-        <v>28602.690000000002</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="53" t="s">
-        <v>214</v>
-      </c>
-      <c r="B15" s="54">
-        <v>23677.59</v>
-      </c>
-      <c r="C15" s="54">
-        <v>45681.2</v>
-      </c>
-      <c r="D15" s="54">
-        <v>73973.349999999991</v>
-      </c>
-      <c r="E15" s="54">
-        <v>8718.7900000000009</v>
-      </c>
-      <c r="F15" s="54">
-        <v>152050.93</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A16"/>
-      <c r="B16"/>
-      <c r="C16"/>
-    </row>
-    <row r="17" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17"/>
-      <c r="B17"/>
-      <c r="C17"/>
-    </row>
-    <row r="18" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="57" t="s">
+    <row r="1" spans="1:15" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" s="81" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="60" t="s">
+        <v>128</v>
+      </c>
+      <c r="B4" s="61" t="s">
+        <v>235</v>
+      </c>
+      <c r="C4" s="61" t="s">
+        <v>236</v>
+      </c>
+      <c r="D4" s="61" t="s">
+        <v>237</v>
+      </c>
+      <c r="E4" s="61" t="s">
+        <v>238</v>
+      </c>
+      <c r="F4" s="61" t="s">
+        <v>239</v>
+      </c>
+      <c r="G4" s="61" t="s">
+        <v>130</v>
+      </c>
+      <c r="H4" s="61" t="s">
+        <v>131</v>
+      </c>
+      <c r="I4" s="61" t="s">
+        <v>132</v>
+      </c>
+      <c r="J4" s="61" t="s">
+        <v>133</v>
+      </c>
+      <c r="K4" s="61" t="s">
+        <v>134</v>
+      </c>
+      <c r="L4" s="62" t="s">
         <v>135</v>
       </c>
-      <c r="B18"/>
-      <c r="C18"/>
-    </row>
-    <row r="19" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="52" t="s">
-        <v>225</v>
-      </c>
-      <c r="B19" s="52" t="s">
-        <v>215</v>
-      </c>
-      <c r="C19"/>
-      <c r="D19"/>
-      <c r="E19"/>
-      <c r="F19"/>
-    </row>
-    <row r="20" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="52" t="s">
-        <v>213</v>
-      </c>
-      <c r="B20" t="s">
-        <v>62</v>
-      </c>
-      <c r="C20" t="s">
-        <v>67</v>
-      </c>
-      <c r="D20" t="s">
-        <v>69</v>
-      </c>
-      <c r="E20" t="s">
-        <v>71</v>
-      </c>
-      <c r="F20" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="53" t="s">
-        <v>216</v>
-      </c>
-      <c r="B21" s="54">
-        <v>97.3</v>
-      </c>
-      <c r="C21" s="54">
-        <v>230.52</v>
-      </c>
-      <c r="D21" s="54">
-        <v>115.52000000000001</v>
-      </c>
-      <c r="E21" s="54">
-        <v>111.77000000000001</v>
-      </c>
-      <c r="F21" s="54">
-        <v>555.11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="53" t="s">
-        <v>217</v>
-      </c>
-      <c r="B22" s="54">
-        <v>96.259999999999991</v>
-      </c>
-      <c r="C22" s="54">
-        <v>211.82</v>
-      </c>
-      <c r="D22" s="54">
-        <v>95.66</v>
-      </c>
-      <c r="E22" s="54">
-        <v>116.5</v>
-      </c>
-      <c r="F22" s="54">
-        <v>520.24</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="53" t="s">
-        <v>218</v>
-      </c>
-      <c r="B23" s="54">
-        <v>90.740000000000009</v>
-      </c>
-      <c r="C23" s="54">
-        <v>227.65</v>
-      </c>
-      <c r="D23" s="54">
-        <v>113.56</v>
-      </c>
-      <c r="E23" s="54">
-        <v>98.47</v>
-      </c>
-      <c r="F23" s="54">
-        <v>530.41999999999996</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A24" s="53" t="s">
-        <v>219</v>
-      </c>
-      <c r="B24" s="54">
-        <v>85.22999999999999</v>
-      </c>
-      <c r="C24" s="54">
-        <v>202.23000000000002</v>
-      </c>
-      <c r="D24" s="54">
-        <v>129.5</v>
-      </c>
-      <c r="E24" s="54">
-        <v>104.87</v>
-      </c>
-      <c r="F24" s="54">
-        <v>521.83000000000004</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="53" t="s">
-        <v>220</v>
-      </c>
-      <c r="B25" s="54">
-        <v>140.46</v>
-      </c>
-      <c r="C25" s="54">
-        <v>268.7</v>
-      </c>
-      <c r="D25" s="54">
-        <v>159.36000000000001</v>
-      </c>
-      <c r="E25" s="54">
-        <v>109.36999999999999</v>
-      </c>
-      <c r="F25" s="54">
-        <v>677.89</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="53" t="s">
-        <v>221</v>
-      </c>
-      <c r="B26" s="54">
-        <v>109.84</v>
-      </c>
-      <c r="C26" s="54">
-        <v>267.16000000000003</v>
-      </c>
-      <c r="D26" s="54">
-        <v>126.93</v>
-      </c>
-      <c r="E26" s="54">
-        <v>100.7</v>
-      </c>
-      <c r="F26" s="54">
-        <v>604.63</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A27" s="53" t="s">
-        <v>222</v>
-      </c>
-      <c r="B27" s="54">
-        <v>113.63</v>
-      </c>
-      <c r="C27" s="54">
-        <v>261.97000000000003</v>
-      </c>
-      <c r="D27" s="54">
-        <v>120.43</v>
-      </c>
-      <c r="E27" s="54">
-        <v>111.67</v>
-      </c>
-      <c r="F27" s="54">
-        <v>607.70000000000005</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A28" s="53" t="s">
-        <v>223</v>
-      </c>
-      <c r="B28" s="54">
-        <v>115.53999999999999</v>
-      </c>
-      <c r="C28" s="54">
-        <v>222.13</v>
-      </c>
-      <c r="D28" s="54">
-        <v>120.43</v>
-      </c>
-      <c r="E28" s="54">
-        <v>109.13999999999999</v>
-      </c>
-      <c r="F28" s="54">
-        <v>567.24</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A29" s="53" t="s">
-        <v>214</v>
-      </c>
-      <c r="B29" s="54">
-        <v>849</v>
-      </c>
-      <c r="C29" s="54">
-        <v>1892.1800000000003</v>
-      </c>
-      <c r="D29" s="54">
-        <v>981.3900000000001</v>
-      </c>
-      <c r="E29" s="54">
-        <v>862.49</v>
-      </c>
-      <c r="F29" s="54">
-        <v>4585.0599999999995</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A30"/>
-      <c r="B30"/>
-      <c r="C30"/>
-    </row>
-    <row r="31" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A31"/>
-      <c r="B31"/>
-      <c r="C31"/>
-    </row>
-    <row r="32" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A32" s="57" t="s">
-        <v>226</v>
-      </c>
-      <c r="B32"/>
-      <c r="C32"/>
-    </row>
-    <row r="33" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A33" s="52" t="s">
-        <v>227</v>
-      </c>
-      <c r="B33" s="52" t="s">
-        <v>215</v>
-      </c>
-      <c r="C33"/>
-      <c r="D33"/>
-      <c r="E33"/>
-      <c r="F33"/>
-    </row>
-    <row r="34" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A34" s="52" t="s">
-        <v>213</v>
-      </c>
-      <c r="B34" t="s">
-        <v>62</v>
-      </c>
-      <c r="C34" t="s">
-        <v>67</v>
-      </c>
-      <c r="D34" t="s">
-        <v>69</v>
-      </c>
-      <c r="E34" t="s">
-        <v>71</v>
-      </c>
-      <c r="F34" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A35" s="53" t="s">
-        <v>216</v>
-      </c>
-      <c r="B35" s="55">
-        <v>38.029188078108938</v>
-      </c>
-      <c r="C35" s="55">
-        <v>23.623763664757938</v>
-      </c>
-      <c r="D35" s="55">
-        <v>69.62231648199446</v>
-      </c>
-      <c r="E35" s="55">
-        <v>11.993647669320925</v>
-      </c>
-      <c r="F35" s="55">
-        <v>33.379492352866997</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A36" s="53" t="s">
-        <v>217</v>
-      </c>
-      <c r="B36" s="55">
-        <v>23.05298150841471</v>
-      </c>
-      <c r="C36" s="55">
-        <v>22.721272778774431</v>
-      </c>
-      <c r="D36" s="55">
-        <v>62.904035124398909</v>
-      </c>
-      <c r="E36" s="55">
-        <v>8.4084978540772521</v>
-      </c>
-      <c r="F36" s="55">
-        <v>26.966188682146701</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A37" s="53" t="s">
-        <v>218</v>
-      </c>
-      <c r="B37" s="55">
-        <v>26.664315627066337</v>
-      </c>
-      <c r="C37" s="55">
-        <v>22.530990555677576</v>
-      </c>
-      <c r="D37" s="55">
-        <v>54.106111306798176</v>
-      </c>
-      <c r="E37" s="55">
-        <v>9.6113537117903931</v>
-      </c>
-      <c r="F37" s="55">
-        <v>27.599675728667844</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A38" s="53" t="s">
-        <v>219</v>
-      </c>
-      <c r="B38" s="55">
-        <v>28.770503343892994</v>
-      </c>
-      <c r="C38" s="55">
-        <v>24.709489195470503</v>
-      </c>
-      <c r="D38" s="55">
-        <v>46.838532818532819</v>
-      </c>
-      <c r="E38" s="55">
-        <v>9.7985124439782592</v>
-      </c>
-      <c r="F38" s="55">
-        <v>27.867830519517845</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A39" s="53" t="s">
-        <v>220</v>
-      </c>
-      <c r="B39" s="55">
-        <v>29.535882101665958</v>
-      </c>
-      <c r="C39" s="55">
-        <v>28.326870115370305</v>
-      </c>
-      <c r="D39" s="55">
-        <v>71.018072289156621</v>
-      </c>
-      <c r="E39" s="55">
-        <v>10.932796927859561</v>
-      </c>
-      <c r="F39" s="55">
-        <v>35.80698933455281</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A40" s="53" t="s">
-        <v>221</v>
-      </c>
-      <c r="B40" s="55">
-        <v>25.945648215586306</v>
-      </c>
-      <c r="C40" s="55">
-        <v>23.422256325797271</v>
-      </c>
-      <c r="D40" s="55">
-        <v>50.511384227526982</v>
-      </c>
-      <c r="E40" s="55">
-        <v>9.8119165839126108</v>
-      </c>
-      <c r="F40" s="55">
-        <v>27.300712832641441</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A41" s="53" t="s">
-        <v>222</v>
-      </c>
-      <c r="B41" s="55">
-        <v>24.392149960397784</v>
-      </c>
-      <c r="C41" s="55">
-        <v>23.104706645799137</v>
-      </c>
-      <c r="D41" s="55">
-        <v>90.877439176284966</v>
-      </c>
-      <c r="E41" s="55">
-        <v>10.383719888958538</v>
-      </c>
-      <c r="F41" s="55">
-        <v>34.438604574625636</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A42" s="53" t="s">
-        <v>223</v>
-      </c>
-      <c r="B42" s="55">
-        <v>26.973169465120307</v>
-      </c>
-      <c r="C42" s="55">
-        <v>24.196596587583848</v>
-      </c>
-      <c r="D42" s="55">
-        <v>158.01776965872293</v>
-      </c>
-      <c r="E42" s="55">
-        <v>9.907824812167858</v>
-      </c>
-      <c r="F42" s="55">
-        <v>50.424317749100915</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A43" s="53" t="s">
-        <v>214</v>
-      </c>
-      <c r="B43" s="55">
-        <v>27.888798586572442</v>
-      </c>
-      <c r="C43" s="55">
-        <v>24.142100645815944</v>
-      </c>
-      <c r="D43" s="55">
-        <v>75.376099206227906</v>
-      </c>
-      <c r="E43" s="55">
-        <v>10.108859233150529</v>
-      </c>
-      <c r="F43" s="55">
-        <v>33.162255237663196</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A44"/>
-      <c r="B44"/>
-      <c r="C44"/>
-    </row>
-    <row r="45" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A45"/>
-      <c r="B45"/>
-      <c r="C45"/>
-    </row>
-    <row r="46" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A46"/>
-      <c r="B46"/>
-      <c r="C46"/>
-    </row>
-    <row r="47" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A47"/>
-      <c r="B47"/>
-      <c r="C47"/>
-    </row>
-    <row r="48" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A48"/>
-      <c r="B48"/>
-      <c r="C48"/>
-    </row>
-    <row r="49" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A49"/>
-      <c r="B49"/>
-      <c r="C49"/>
-    </row>
-    <row r="50" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A50"/>
-      <c r="B50"/>
-      <c r="C50"/>
+      <c r="M4" s="60" t="s">
+        <v>136</v>
+      </c>
+      <c r="N4" s="61" t="s">
+        <v>120</v>
+      </c>
+      <c r="O4" s="61" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A5" s="70" t="s">
+        <v>138</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>240</v>
+      </c>
+      <c r="C5" s="77">
+        <v>0</v>
+      </c>
+      <c r="D5" s="77">
+        <v>0</v>
+      </c>
+      <c r="E5" s="77">
+        <v>0</v>
+      </c>
+      <c r="F5" s="77">
+        <v>0</v>
+      </c>
+      <c r="G5" s="42">
+        <v>1558</v>
+      </c>
+      <c r="H5" s="42">
+        <v>2687</v>
+      </c>
+      <c r="I5" s="42">
+        <v>9515</v>
+      </c>
+      <c r="J5" s="42">
+        <v>1298</v>
+      </c>
+      <c r="K5" s="42">
+        <f>SUM(G5:J5)</f>
+        <v>15058</v>
+      </c>
+      <c r="L5" s="78">
+        <v>470</v>
+      </c>
+      <c r="M5" s="79">
+        <v>-56843.21</v>
+      </c>
+      <c r="N5" s="80">
+        <v>-97563.64</v>
+      </c>
+      <c r="O5" s="77">
+        <f>M5-N5</f>
+        <v>40720.43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A6" s="70" t="s">
+        <v>241</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>242</v>
+      </c>
+      <c r="C6" s="77">
+        <v>-220.92</v>
+      </c>
+      <c r="D6" s="77">
+        <v>-87.43</v>
+      </c>
+      <c r="E6" s="77">
+        <v>-87.67</v>
+      </c>
+      <c r="F6" s="77">
+        <v>-98.15</v>
+      </c>
+      <c r="G6" s="42">
+        <v>1558</v>
+      </c>
+      <c r="H6" s="42">
+        <v>2687</v>
+      </c>
+      <c r="I6" s="42">
+        <v>9515</v>
+      </c>
+      <c r="J6" s="42">
+        <v>541</v>
+      </c>
+      <c r="K6" s="42">
+        <f>SUM(G6:J6)</f>
+        <v>14301</v>
+      </c>
+      <c r="L6" s="78">
+        <v>435</v>
+      </c>
+      <c r="M6" s="79">
+        <v>-106047.83</v>
+      </c>
+      <c r="N6" s="80">
+        <v>-171192.31</v>
+      </c>
+      <c r="O6" s="77">
+        <f>M6-N6</f>
+        <v>65144.479999999996</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7" s="70" t="s">
+        <v>243</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>244</v>
+      </c>
+      <c r="C7" s="77">
+        <v>206.55</v>
+      </c>
+      <c r="D7" s="77">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="E7" s="77">
+        <v>83.55</v>
+      </c>
+      <c r="F7" s="77">
+        <v>76.150000000000006</v>
+      </c>
+      <c r="G7" s="42">
+        <v>1558</v>
+      </c>
+      <c r="H7" s="42">
+        <v>8062</v>
+      </c>
+      <c r="I7" s="42">
+        <v>9515</v>
+      </c>
+      <c r="J7" s="42">
+        <v>1298</v>
+      </c>
+      <c r="K7" s="42">
+        <f>SUM(G7:J7)</f>
+        <v>20433</v>
+      </c>
+      <c r="L7" s="78">
+        <v>630</v>
+      </c>
+      <c r="M7" s="79">
+        <v>-9141.3799999999992</v>
+      </c>
+      <c r="N7" s="80">
+        <v>-30804.68</v>
+      </c>
+      <c r="O7" s="77">
+        <f>M7-N7</f>
+        <v>21663.300000000003</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A8" s="70" t="s">
+        <v>245</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>246</v>
+      </c>
+      <c r="C8" s="77">
+        <v>206.55</v>
+      </c>
+      <c r="D8" s="77">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="E8" s="77">
+        <v>83.55</v>
+      </c>
+      <c r="F8" s="77">
+        <v>-98.15</v>
+      </c>
+      <c r="G8" s="42">
+        <v>1558</v>
+      </c>
+      <c r="H8" s="42">
+        <v>8062</v>
+      </c>
+      <c r="I8" s="42">
+        <v>9515</v>
+      </c>
+      <c r="J8" s="42">
+        <v>541</v>
+      </c>
+      <c r="K8" s="42">
+        <f>SUM(G8:J8)</f>
+        <v>19676</v>
+      </c>
+      <c r="L8" s="78">
+        <v>595</v>
+      </c>
+      <c r="M8" s="79">
+        <v>-26881.35</v>
+      </c>
+      <c r="N8" s="80">
+        <v>-49473.09</v>
+      </c>
+      <c r="O8" s="77">
+        <f>M8-N8</f>
+        <v>22591.739999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A9" s="70" t="s">
+        <v>247</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>248</v>
+      </c>
+      <c r="C9" s="77">
+        <v>-220.92</v>
+      </c>
+      <c r="D9" s="77">
+        <v>-87.43</v>
+      </c>
+      <c r="E9" s="77">
+        <v>-87.67</v>
+      </c>
+      <c r="F9" s="77">
+        <v>76.150000000000006</v>
+      </c>
+      <c r="G9" s="42">
+        <v>1558</v>
+      </c>
+      <c r="H9" s="42">
+        <v>2687</v>
+      </c>
+      <c r="I9" s="42">
+        <v>9515</v>
+      </c>
+      <c r="J9" s="42">
+        <v>1298</v>
+      </c>
+      <c r="K9" s="42">
+        <f>SUM(G9:J9)</f>
+        <v>15058</v>
+      </c>
+      <c r="L9" s="78">
+        <v>470</v>
+      </c>
+      <c r="M9" s="79">
+        <v>-88307.85</v>
+      </c>
+      <c r="N9" s="80">
+        <v>-152523.89000000001</v>
+      </c>
+      <c r="O9" s="77">
+        <f>M9-N9</f>
+        <v>64216.040000000008</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="88" t="s">
+        <v>250</v>
+      </c>
+      <c r="B11" s="87"/>
+      <c r="C11" s="87"/>
+      <c r="D11" s="87"/>
+      <c r="E11" s="87"/>
+      <c r="F11" s="87"/>
+      <c r="G11" s="87"/>
+      <c r="H11" s="87"/>
+      <c r="I11" s="87"/>
+      <c r="J11" s="87"/>
+      <c r="K11" s="87"/>
+      <c r="L11" s="87"/>
+      <c r="M11" s="87"/>
+      <c r="N11" s="87"/>
+      <c r="O11" s="87"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A11:O11"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId4"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:B14"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{688C7ABA-8B71-48C7-A456-D4978829B4A9}">
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="120" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="41" t="s">
-        <v>157</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="41" t="s">
-        <v>159</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="41" t="s">
-        <v>161</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="41" t="s">
-        <v>163</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="41" t="s">
-        <v>165</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="41" t="s">
-        <v>167</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="41" t="s">
-        <v>168</v>
-      </c>
-      <c r="B10" s="19" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="41" t="s">
-        <v>170</v>
-      </c>
-      <c r="B11" s="19" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="41" t="s">
-        <v>172</v>
-      </c>
-      <c r="B12" s="19" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="46" t="s">
-        <v>205</v>
-      </c>
-      <c r="B13" s="47" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="46" t="s">
-        <v>207</v>
-      </c>
-      <c r="B14" s="47" t="s">
-        <v>208</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:Q9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF1ED514-E10E-4E95-8B6A-02C8F94ECDA5}">
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="17" width="14" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:17" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A2" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B2" s="15">
-        <v>23677.59</v>
-      </c>
-      <c r="C2" s="15">
-        <v>846</v>
-      </c>
-      <c r="D2" s="15">
-        <v>1368</v>
-      </c>
-      <c r="E2" s="15">
-        <v>3420</v>
-      </c>
-      <c r="F2" s="15">
-        <v>32.03</v>
-      </c>
-      <c r="G2" s="15">
-        <v>27.99</v>
-      </c>
-      <c r="H2" s="15">
-        <v>382</v>
-      </c>
-      <c r="I2" s="15">
-        <v>251.54</v>
-      </c>
-      <c r="J2" s="15">
-        <v>321.20999999999998</v>
-      </c>
-      <c r="K2" s="15">
-        <v>7.8529999999999998</v>
-      </c>
-      <c r="L2" s="15">
-        <v>11.477</v>
-      </c>
-      <c r="M2" s="15">
-        <v>3</v>
-      </c>
-      <c r="N2" s="15">
-        <v>1</v>
-      </c>
-      <c r="O2" s="15">
-        <v>742.49</v>
-      </c>
-      <c r="P2" s="15">
-        <v>-490.95</v>
-      </c>
-      <c r="Q2" s="15">
-        <v>-15.327999999999999</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="B3" s="15">
-        <v>0</v>
-      </c>
-      <c r="C3" s="15">
-        <v>1401</v>
-      </c>
-      <c r="D3" s="15">
-        <v>1831</v>
-      </c>
-      <c r="E3" s="15">
-        <v>4577.5</v>
-      </c>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15">
-        <v>650</v>
-      </c>
-      <c r="I3" s="15">
-        <v>167.97</v>
-      </c>
-      <c r="J3" s="15">
-        <v>217.02</v>
-      </c>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
-      <c r="M3" s="15"/>
-      <c r="N3" s="15"/>
-      <c r="O3" s="15">
-        <v>196.21</v>
-      </c>
-      <c r="P3" s="15">
-        <v>-28.24</v>
-      </c>
-      <c r="Q3" s="15"/>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A4" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="B4" s="15">
-        <v>45681.2</v>
-      </c>
-      <c r="C4" s="15">
-        <v>1545</v>
-      </c>
-      <c r="D4" s="15">
-        <v>2086</v>
-      </c>
-      <c r="E4" s="15">
-        <v>5215</v>
-      </c>
-      <c r="F4" s="15">
-        <v>32.94</v>
-      </c>
-      <c r="G4" s="15">
-        <v>29.57</v>
-      </c>
-      <c r="H4" s="15">
-        <v>719</v>
-      </c>
-      <c r="I4" s="15">
-        <v>185.36</v>
-      </c>
-      <c r="J4" s="15">
-        <v>237.31</v>
-      </c>
-      <c r="K4" s="15">
-        <v>5.6269999999999998</v>
-      </c>
-      <c r="L4" s="15">
-        <v>8.0259999999999998</v>
-      </c>
-      <c r="M4" s="15">
-        <v>4</v>
-      </c>
-      <c r="N4" s="15">
-        <v>1</v>
-      </c>
-      <c r="O4" s="15">
-        <v>217.32</v>
-      </c>
-      <c r="P4" s="15">
-        <v>-31.96</v>
-      </c>
-      <c r="Q4" s="15">
-        <v>-0.97</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A5" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="B5" s="15">
-        <v>73973.350000000006</v>
-      </c>
-      <c r="C5" s="15">
-        <v>1225</v>
-      </c>
-      <c r="D5" s="15">
-        <v>2550</v>
-      </c>
-      <c r="E5" s="15">
-        <v>6375</v>
-      </c>
-      <c r="F5" s="15">
-        <v>65.59</v>
-      </c>
-      <c r="G5" s="15">
-        <v>60.39</v>
-      </c>
-      <c r="H5" s="15">
-        <v>562</v>
-      </c>
-      <c r="I5" s="15">
-        <v>171.28</v>
-      </c>
-      <c r="J5" s="15">
-        <v>216.32</v>
-      </c>
-      <c r="K5" s="15">
-        <v>2.6110000000000002</v>
-      </c>
-      <c r="L5" s="15">
-        <v>3.5819999999999999</v>
-      </c>
-      <c r="M5" s="15">
-        <v>6</v>
-      </c>
-      <c r="N5" s="15">
-        <v>1</v>
-      </c>
-      <c r="O5" s="15">
-        <v>225.31</v>
-      </c>
-      <c r="P5" s="15">
-        <v>-54.03</v>
-      </c>
-      <c r="Q5" s="15">
-        <v>-0.82399999999999995</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A6" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="15">
-        <v>8718.7900000000009</v>
-      </c>
-      <c r="C6" s="15">
-        <v>911</v>
-      </c>
-      <c r="D6" s="15">
-        <v>1056</v>
-      </c>
-      <c r="E6" s="15">
-        <v>2640</v>
-      </c>
-      <c r="F6" s="15">
-        <v>12.47</v>
-      </c>
-      <c r="G6" s="15">
-        <v>9.57</v>
-      </c>
-      <c r="H6" s="15">
-        <v>467</v>
-      </c>
-      <c r="I6" s="15">
-        <v>165.36</v>
-      </c>
-      <c r="J6" s="15">
-        <v>217.06</v>
-      </c>
-      <c r="K6" s="15">
-        <v>13.262</v>
-      </c>
-      <c r="L6" s="15">
-        <v>22.68</v>
-      </c>
-      <c r="M6" s="15">
-        <v>2</v>
-      </c>
-      <c r="N6" s="15">
-        <v>1</v>
-      </c>
-      <c r="O6" s="15">
-        <v>110.87</v>
-      </c>
-      <c r="P6" s="15">
-        <v>54.49</v>
-      </c>
-      <c r="Q6" s="15">
-        <v>4.3710000000000004</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>191</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Point the assumptions, business questions and descriptions to the checks added later
</commit_message>
<xml_diff>
--- a/excel/budget_model.xlsx
+++ b/excel/budget_model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40576ae3754c8ac9/Υπολογιστής/Ο Φάκελός μου/Data analyst projects/FinTech Customer Acquisition and Profitability Analysis/FinTech-Customer-Acquisition-and-Profitability-Analysis/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3986" documentId="8_{DA684D4A-D9C9-4D3B-8B67-0B4778129DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3F7502A0-37FF-471B-BEB2-74E437448CCE}"/>
+  <xr:revisionPtr revIDLastSave="3988" documentId="8_{DA684D4A-D9C9-4D3B-8B67-0B4778129DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{980DA29E-DB2B-49DD-95AD-9A9745B27369}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -129,9 +129,6 @@
     <t>What the model says (at the delivered inputs)</t>
   </si>
   <si>
-    <t>1. After credit losses, only referral earns money per customer. Affiliate looks best before losses but loses the most per customer, because its borrowers default far more often.</t>
-  </si>
-  <si>
     <t>2. The best allocation puts affiliate, paid search and paid social at their lower limit (50 percent of baseline) and referral at its upper limit (120 percent). The model never wants more spend in a channel whose customers lose money.</t>
   </si>
   <si>
@@ -702,9 +699,6 @@
     <t>Sheets look up values by channel name with VLOOKUP (exact match). SUMIFS adds up the data sheets by channel and month, and COUNTIF finds the payback month.</t>
   </si>
   <si>
-    <t>Sheets: Assumptions (inputs) &gt; Unit_Economics (CAC, LTV, payback) &gt; Curves (spend to customers) &gt; Optimizer (Solver) &gt; Scenarios &gt; Pivot_Tables. Data_ sheets hold the SQL view results.</t>
-  </si>
-  <si>
     <t>quarter</t>
   </si>
   <si>
@@ -826,6 +820,12 @@
   </si>
   <si>
     <t>Reading: affiliate and paid social stay at their lower limit in all five cases, even when their value is at the high end of its interval, so cutting them does not depend on the point estimates. Referral and paid search are the two swing channels: referral falls to its lower limit when its value is at the low end (the interval includes zero), and paid search rises to its upper limit when its value is at the high end. Net profit stays negative in every case, and the uplift is positive in every case.</t>
+  </si>
+  <si>
+    <t>1. After credit losses, only referral has a positive average value per customer (+54 EUR), but its 95% bootstrap interval (-44 to +131) includes zero, so it is not proven. Affiliate looks best before losses and is clearly the worst after them, because its borrowers default far more often.</t>
+  </si>
+  <si>
+    <t>Sheets: Assumptions (inputs) &gt; Unit_Economics (CAC, LTV, payback) &gt; Curves (spend to customers) &gt; Optimizer (Solver) &gt; Scenarios &gt; LTV_Scenarios (values moved within their bootstrap intervals) &gt; Pivot_Tables. Data_ sheets hold the SQL view results.</t>
   </si>
 </sst>
 </file>
@@ -1253,16 +1253,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6300,7 +6300,7 @@
     </row>
     <row r="21" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="84" t="s">
-        <v>18</v>
+        <v>249</v>
       </c>
       <c r="B21" s="83"/>
       <c r="C21" s="83"/>
@@ -6311,7 +6311,7 @@
     </row>
     <row r="22" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="84" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B22" s="83"/>
       <c r="C22" s="83"/>
@@ -6322,7 +6322,7 @@
     </row>
     <row r="23" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="84" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B23" s="83"/>
       <c r="C23" s="83"/>
@@ -6333,7 +6333,7 @@
     </row>
     <row r="24" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="84" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B24" s="83"/>
       <c r="C24" s="83"/>
@@ -6344,7 +6344,7 @@
     </row>
     <row r="25" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="84" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B25" s="83"/>
       <c r="C25" s="83"/>
@@ -6355,7 +6355,7 @@
     </row>
     <row r="27" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="82" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B27" s="83"/>
       <c r="C27" s="83"/>
@@ -6366,32 +6366,32 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>209</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -6437,25 +6437,25 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="51" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="50" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="56" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" s="52" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B5" s="52" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C5"/>
       <c r="D5"/>
@@ -6464,27 +6464,27 @@
     </row>
     <row r="6" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" s="52" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" s="53" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B7" s="54">
         <v>3700.24</v>
@@ -6504,7 +6504,7 @@
     </row>
     <row r="8" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" s="53" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B8" s="54">
         <v>2219.08</v>
@@ -6524,7 +6524,7 @@
     </row>
     <row r="9" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="53" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B9" s="54">
         <v>2419.5199999999995</v>
@@ -6544,7 +6544,7 @@
     </row>
     <row r="10" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A10" s="53" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B10" s="54">
         <v>2452.1099999999997</v>
@@ -6564,7 +6564,7 @@
     </row>
     <row r="11" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" s="53" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B11" s="54">
         <v>4148.6100000000006</v>
@@ -6584,7 +6584,7 @@
     </row>
     <row r="12" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A12" s="53" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B12" s="54">
         <v>2849.87</v>
@@ -6604,7 +6604,7 @@
     </row>
     <row r="13" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" s="53" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B13" s="54">
         <v>2771.6800000000003</v>
@@ -6624,7 +6624,7 @@
     </row>
     <row r="14" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A14" s="53" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B14" s="54">
         <v>3116.48</v>
@@ -6644,7 +6644,7 @@
     </row>
     <row r="15" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A15" s="53" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B15" s="54">
         <v>23677.59</v>
@@ -6674,17 +6674,17 @@
     </row>
     <row r="18" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A18" s="57" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
     </row>
     <row r="19" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A19" s="52" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B19" s="52" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C19"/>
       <c r="D19"/>
@@ -6693,27 +6693,27 @@
     </row>
     <row r="20" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A20" s="52" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F20" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A21" s="53" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B21" s="54">
         <v>97.3</v>
@@ -6733,7 +6733,7 @@
     </row>
     <row r="22" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A22" s="53" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B22" s="54">
         <v>96.259999999999991</v>
@@ -6753,7 +6753,7 @@
     </row>
     <row r="23" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A23" s="53" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B23" s="54">
         <v>90.740000000000009</v>
@@ -6773,7 +6773,7 @@
     </row>
     <row r="24" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A24" s="53" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B24" s="54">
         <v>85.22999999999999</v>
@@ -6793,7 +6793,7 @@
     </row>
     <row r="25" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A25" s="53" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B25" s="54">
         <v>140.46</v>
@@ -6813,7 +6813,7 @@
     </row>
     <row r="26" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A26" s="53" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B26" s="54">
         <v>109.84</v>
@@ -6833,7 +6833,7 @@
     </row>
     <row r="27" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A27" s="53" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B27" s="54">
         <v>113.63</v>
@@ -6853,7 +6853,7 @@
     </row>
     <row r="28" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A28" s="53" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B28" s="54">
         <v>115.53999999999999</v>
@@ -6873,7 +6873,7 @@
     </row>
     <row r="29" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A29" s="53" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B29" s="54">
         <v>849</v>
@@ -6903,17 +6903,17 @@
     </row>
     <row r="32" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A32" s="57" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B32"/>
       <c r="C32"/>
     </row>
     <row r="33" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A33" s="52" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B33" s="52" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -6922,27 +6922,27 @@
     </row>
     <row r="34" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A34" s="52" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B34" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C34" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D34" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E34" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F34" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A35" s="53" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B35" s="55">
         <v>38.029188078108938</v>
@@ -6962,7 +6962,7 @@
     </row>
     <row r="36" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A36" s="53" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B36" s="55">
         <v>23.05298150841471</v>
@@ -6982,7 +6982,7 @@
     </row>
     <row r="37" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A37" s="53" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B37" s="55">
         <v>26.664315627066337</v>
@@ -7002,7 +7002,7 @@
     </row>
     <row r="38" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A38" s="53" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B38" s="55">
         <v>28.770503343892994</v>
@@ -7022,7 +7022,7 @@
     </row>
     <row r="39" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A39" s="53" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B39" s="55">
         <v>29.535882101665958</v>
@@ -7042,7 +7042,7 @@
     </row>
     <row r="40" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A40" s="53" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B40" s="55">
         <v>25.945648215586306</v>
@@ -7062,7 +7062,7 @@
     </row>
     <row r="41" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A41" s="53" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B41" s="55">
         <v>24.392149960397784</v>
@@ -7082,7 +7082,7 @@
     </row>
     <row r="42" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A42" s="53" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B42" s="55">
         <v>26.973169465120307</v>
@@ -7102,7 +7102,7 @@
     </row>
     <row r="43" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A43" s="53" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B43" s="55">
         <v>27.888798586572442</v>
@@ -7172,103 +7172,103 @@
   <sheetData>
     <row r="1" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="41" t="s">
+        <v>156</v>
+      </c>
+      <c r="B4" s="19" t="s">
         <v>157</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="41" t="s">
+        <v>158</v>
+      </c>
+      <c r="B5" s="19" t="s">
         <v>159</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="41" t="s">
+        <v>160</v>
+      </c>
+      <c r="B6" s="19" t="s">
         <v>161</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="41" t="s">
+        <v>162</v>
+      </c>
+      <c r="B7" s="19" t="s">
         <v>163</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="41" t="s">
+        <v>164</v>
+      </c>
+      <c r="B8" s="19" t="s">
         <v>165</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="41" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="41" t="s">
+        <v>167</v>
+      </c>
+      <c r="B10" s="19" t="s">
         <v>168</v>
-      </c>
-      <c r="B10" s="19" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="41" t="s">
+        <v>169</v>
+      </c>
+      <c r="B11" s="19" t="s">
         <v>170</v>
-      </c>
-      <c r="B11" s="19" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="41" t="s">
+        <v>171</v>
+      </c>
+      <c r="B12" s="19" t="s">
         <v>172</v>
-      </c>
-      <c r="B12" s="19" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="46" t="s">
+        <v>204</v>
+      </c>
+      <c r="B13" s="47" t="s">
         <v>205</v>
-      </c>
-      <c r="B13" s="47" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="46" t="s">
+        <v>206</v>
+      </c>
+      <c r="B14" s="47" t="s">
         <v>207</v>
-      </c>
-      <c r="B14" s="47" t="s">
-        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -7287,60 +7287,60 @@
   <sheetData>
     <row r="1" spans="1:17" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="Q1" s="5" t="s">
         <v>189</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B2" s="15">
         <v>23677.59</v>
@@ -7393,7 +7393,7 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B3" s="15">
         <v>0</v>
@@ -7432,7 +7432,7 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B4" s="15">
         <v>45681.2</v>
@@ -7485,7 +7485,7 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B5" s="15">
         <v>73973.350000000006</v>
@@ -7538,7 +7538,7 @@
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6" s="15">
         <v>8718.7900000000009</v>
@@ -7591,7 +7591,7 @@
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -7614,37 +7614,37 @@
   <sheetData>
     <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="C1" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="G1" s="5" t="s">
-        <v>197</v>
-      </c>
       <c r="H1" s="5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="I1" s="2"/>
       <c r="J1" s="50" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B2" s="43">
         <v>45566</v>
@@ -7673,7 +7673,7 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B3" s="43">
         <v>45597</v>
@@ -7702,7 +7702,7 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B4" s="43">
         <v>45627</v>
@@ -7731,7 +7731,7 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B5" s="43">
         <v>45658</v>
@@ -7760,7 +7760,7 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B6" s="43">
         <v>45689</v>
@@ -7789,7 +7789,7 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B7" s="43">
         <v>45717</v>
@@ -7818,7 +7818,7 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B8" s="43">
         <v>45748</v>
@@ -7847,7 +7847,7 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B9" s="43">
         <v>45778</v>
@@ -7876,7 +7876,7 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B10" s="43">
         <v>45809</v>
@@ -7905,7 +7905,7 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B11" s="43">
         <v>45839</v>
@@ -7934,7 +7934,7 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B12" s="43">
         <v>45870</v>
@@ -7963,7 +7963,7 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B13" s="43">
         <v>45901</v>
@@ -7992,7 +7992,7 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B14" s="43">
         <v>45931</v>
@@ -8021,7 +8021,7 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B15" s="43">
         <v>45962</v>
@@ -8050,7 +8050,7 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B16" s="43">
         <v>45992</v>
@@ -8079,7 +8079,7 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B17" s="43">
         <v>46023</v>
@@ -8108,7 +8108,7 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B18" s="43">
         <v>46054</v>
@@ -8137,7 +8137,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B19" s="43">
         <v>46082</v>
@@ -8166,7 +8166,7 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B20" s="43">
         <v>46113</v>
@@ -8195,7 +8195,7 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B21" s="43">
         <v>46143</v>
@@ -8224,7 +8224,7 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B22" s="43">
         <v>46174</v>
@@ -8253,7 +8253,7 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B23" s="43">
         <v>46204</v>
@@ -8282,7 +8282,7 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B24" s="43">
         <v>46235</v>
@@ -8311,7 +8311,7 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B25" s="43">
         <v>46266</v>
@@ -8340,7 +8340,7 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B26" s="43">
         <v>45566</v>
@@ -8369,7 +8369,7 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B27" s="43">
         <v>45597</v>
@@ -8398,7 +8398,7 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B28" s="43">
         <v>45627</v>
@@ -8427,7 +8427,7 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B29" s="43">
         <v>45658</v>
@@ -8456,7 +8456,7 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B30" s="43">
         <v>45689</v>
@@ -8485,7 +8485,7 @@
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B31" s="43">
         <v>45717</v>
@@ -8514,7 +8514,7 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B32" s="43">
         <v>45748</v>
@@ -8543,7 +8543,7 @@
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B33" s="43">
         <v>45778</v>
@@ -8572,7 +8572,7 @@
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B34" s="43">
         <v>45809</v>
@@ -8601,7 +8601,7 @@
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B35" s="43">
         <v>45839</v>
@@ -8630,7 +8630,7 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B36" s="43">
         <v>45870</v>
@@ -8659,7 +8659,7 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B37" s="43">
         <v>45901</v>
@@ -8688,7 +8688,7 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B38" s="43">
         <v>45931</v>
@@ -8717,7 +8717,7 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B39" s="43">
         <v>45962</v>
@@ -8746,7 +8746,7 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B40" s="43">
         <v>45992</v>
@@ -8775,7 +8775,7 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B41" s="43">
         <v>46023</v>
@@ -8804,7 +8804,7 @@
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B42" s="43">
         <v>46054</v>
@@ -8833,7 +8833,7 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B43" s="43">
         <v>46082</v>
@@ -8862,7 +8862,7 @@
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B44" s="43">
         <v>46113</v>
@@ -8891,7 +8891,7 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B45" s="43">
         <v>46143</v>
@@ -8920,7 +8920,7 @@
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B46" s="43">
         <v>46174</v>
@@ -8949,7 +8949,7 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B47" s="43">
         <v>46204</v>
@@ -8978,7 +8978,7 @@
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B48" s="43">
         <v>46235</v>
@@ -9007,7 +9007,7 @@
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B49" s="43">
         <v>46266</v>
@@ -9036,7 +9036,7 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B50" s="43">
         <v>45566</v>
@@ -9065,7 +9065,7 @@
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B51" s="43">
         <v>45597</v>
@@ -9094,7 +9094,7 @@
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B52" s="43">
         <v>45627</v>
@@ -9123,7 +9123,7 @@
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B53" s="43">
         <v>45658</v>
@@ -9152,7 +9152,7 @@
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B54" s="43">
         <v>45689</v>
@@ -9181,7 +9181,7 @@
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B55" s="43">
         <v>45717</v>
@@ -9210,7 +9210,7 @@
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B56" s="43">
         <v>45748</v>
@@ -9239,7 +9239,7 @@
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B57" s="43">
         <v>45778</v>
@@ -9268,7 +9268,7 @@
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B58" s="43">
         <v>45809</v>
@@ -9297,7 +9297,7 @@
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B59" s="43">
         <v>45839</v>
@@ -9326,7 +9326,7 @@
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B60" s="43">
         <v>45870</v>
@@ -9355,7 +9355,7 @@
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B61" s="43">
         <v>45901</v>
@@ -9384,7 +9384,7 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B62" s="43">
         <v>45931</v>
@@ -9413,7 +9413,7 @@
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B63" s="43">
         <v>45962</v>
@@ -9442,7 +9442,7 @@
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B64" s="43">
         <v>45992</v>
@@ -9471,7 +9471,7 @@
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B65" s="43">
         <v>46023</v>
@@ -9500,7 +9500,7 @@
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B66" s="43">
         <v>46054</v>
@@ -9529,7 +9529,7 @@
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B67" s="43">
         <v>46082</v>
@@ -9558,7 +9558,7 @@
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B68" s="43">
         <v>46113</v>
@@ -9587,7 +9587,7 @@
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B69" s="43">
         <v>46143</v>
@@ -9616,7 +9616,7 @@
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B70" s="43">
         <v>46174</v>
@@ -9645,7 +9645,7 @@
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B71" s="43">
         <v>46204</v>
@@ -9674,7 +9674,7 @@
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B72" s="43">
         <v>46235</v>
@@ -9703,7 +9703,7 @@
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B73" s="43">
         <v>46266</v>
@@ -9732,7 +9732,7 @@
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B74" s="43">
         <v>45566</v>
@@ -9761,7 +9761,7 @@
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B75" s="43">
         <v>45597</v>
@@ -9790,7 +9790,7 @@
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B76" s="43">
         <v>45627</v>
@@ -9819,7 +9819,7 @@
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B77" s="43">
         <v>45658</v>
@@ -9848,7 +9848,7 @@
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B78" s="43">
         <v>45689</v>
@@ -9877,7 +9877,7 @@
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B79" s="43">
         <v>45717</v>
@@ -9906,7 +9906,7 @@
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B80" s="43">
         <v>45748</v>
@@ -9935,7 +9935,7 @@
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A81" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B81" s="43">
         <v>45778</v>
@@ -9964,7 +9964,7 @@
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A82" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B82" s="43">
         <v>45809</v>
@@ -9993,7 +9993,7 @@
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A83" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B83" s="43">
         <v>45839</v>
@@ -10022,7 +10022,7 @@
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A84" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B84" s="43">
         <v>45870</v>
@@ -10051,7 +10051,7 @@
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A85" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B85" s="43">
         <v>45901</v>
@@ -10080,7 +10080,7 @@
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A86" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B86" s="43">
         <v>45931</v>
@@ -10109,7 +10109,7 @@
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A87" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B87" s="43">
         <v>45962</v>
@@ -10138,7 +10138,7 @@
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A88" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B88" s="43">
         <v>45992</v>
@@ -10167,7 +10167,7 @@
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A89" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B89" s="43">
         <v>46023</v>
@@ -10196,7 +10196,7 @@
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A90" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B90" s="43">
         <v>46054</v>
@@ -10225,7 +10225,7 @@
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A91" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B91" s="43">
         <v>46082</v>
@@ -10254,7 +10254,7 @@
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A92" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B92" s="43">
         <v>46113</v>
@@ -10283,7 +10283,7 @@
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A93" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B93" s="43">
         <v>46143</v>
@@ -10312,7 +10312,7 @@
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A94" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B94" s="43">
         <v>46174</v>
@@ -10341,7 +10341,7 @@
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A95" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B95" s="43">
         <v>46204</v>
@@ -10370,7 +10370,7 @@
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A96" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B96" s="43">
         <v>46235</v>
@@ -10399,7 +10399,7 @@
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A97" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B97" s="43">
         <v>46266</v>
@@ -10444,27 +10444,27 @@
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>201</v>
-      </c>
       <c r="G1" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B2" s="15">
         <v>1</v>
@@ -10481,7 +10481,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B3" s="15">
         <v>2</v>
@@ -10498,7 +10498,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B4" s="15">
         <v>3</v>
@@ -10515,7 +10515,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B5" s="15">
         <v>4</v>
@@ -10532,7 +10532,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B6" s="15">
         <v>5</v>
@@ -10549,7 +10549,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B7" s="15">
         <v>6</v>
@@ -10566,7 +10566,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B8" s="15">
         <v>7</v>
@@ -10583,7 +10583,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B9" s="15">
         <v>8</v>
@@ -10600,7 +10600,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B10" s="15">
         <v>9</v>
@@ -10617,7 +10617,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B11" s="15">
         <v>10</v>
@@ -10634,7 +10634,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B12" s="15">
         <v>11</v>
@@ -10651,7 +10651,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B13" s="15">
         <v>12</v>
@@ -10668,7 +10668,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B14" s="15">
         <v>1</v>
@@ -10685,7 +10685,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B15" s="15">
         <v>2</v>
@@ -10702,7 +10702,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B16" s="15">
         <v>3</v>
@@ -10719,7 +10719,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B17" s="15">
         <v>4</v>
@@ -10736,7 +10736,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B18" s="15">
         <v>5</v>
@@ -10753,7 +10753,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B19" s="15">
         <v>6</v>
@@ -10770,7 +10770,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B20" s="15">
         <v>7</v>
@@ -10787,7 +10787,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B21" s="15">
         <v>8</v>
@@ -10804,7 +10804,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B22" s="15">
         <v>9</v>
@@ -10821,7 +10821,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B23" s="15">
         <v>10</v>
@@ -10838,7 +10838,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B24" s="15">
         <v>11</v>
@@ -10855,7 +10855,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B25" s="15">
         <v>12</v>
@@ -10872,7 +10872,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B26" s="15">
         <v>1</v>
@@ -10889,7 +10889,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B27" s="15">
         <v>2</v>
@@ -10906,7 +10906,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B28" s="15">
         <v>3</v>
@@ -10923,7 +10923,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B29" s="15">
         <v>4</v>
@@ -10940,7 +10940,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B30" s="15">
         <v>5</v>
@@ -10957,7 +10957,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B31" s="15">
         <v>6</v>
@@ -10974,7 +10974,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B32" s="15">
         <v>7</v>
@@ -10991,7 +10991,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B33" s="15">
         <v>8</v>
@@ -11008,7 +11008,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B34" s="15">
         <v>9</v>
@@ -11025,7 +11025,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B35" s="15">
         <v>10</v>
@@ -11042,7 +11042,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B36" s="15">
         <v>11</v>
@@ -11059,7 +11059,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B37" s="15">
         <v>12</v>
@@ -11076,7 +11076,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B38" s="15">
         <v>1</v>
@@ -11093,7 +11093,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B39" s="15">
         <v>2</v>
@@ -11110,7 +11110,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B40" s="15">
         <v>3</v>
@@ -11127,7 +11127,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B41" s="15">
         <v>4</v>
@@ -11144,7 +11144,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B42" s="15">
         <v>5</v>
@@ -11161,7 +11161,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B43" s="15">
         <v>6</v>
@@ -11178,7 +11178,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B44" s="15">
         <v>7</v>
@@ -11195,7 +11195,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B45" s="15">
         <v>8</v>
@@ -11212,7 +11212,7 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B46" s="15">
         <v>9</v>
@@ -11229,7 +11229,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B47" s="15">
         <v>10</v>
@@ -11246,7 +11246,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B48" s="15">
         <v>11</v>
@@ -11263,7 +11263,7 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B49" s="15">
         <v>12</v>
@@ -11280,7 +11280,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B50" s="15">
         <v>1</v>
@@ -11297,7 +11297,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B51" s="15">
         <v>2</v>
@@ -11314,7 +11314,7 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B52" s="15">
         <v>3</v>
@@ -11331,7 +11331,7 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B53" s="15">
         <v>4</v>
@@ -11348,7 +11348,7 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B54" s="15">
         <v>5</v>
@@ -11365,7 +11365,7 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B55" s="15">
         <v>6</v>
@@ -11382,7 +11382,7 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B56" s="15">
         <v>7</v>
@@ -11399,7 +11399,7 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B57" s="15">
         <v>8</v>
@@ -11416,7 +11416,7 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B58" s="15">
         <v>9</v>
@@ -11433,7 +11433,7 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B59" s="15">
         <v>10</v>
@@ -11450,7 +11450,7 @@
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B60" s="15">
         <v>11</v>
@@ -11467,7 +11467,7 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B61" s="15">
         <v>12</v>
@@ -11499,157 +11499,157 @@
   <sheetData>
     <row r="1" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>33</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B5" s="20">
         <v>2.5</v>
       </c>
       <c r="C5" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="19" t="s">
         <v>36</v>
-      </c>
-      <c r="D5" s="19" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B6" s="21">
         <v>3</v>
       </c>
       <c r="C6" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="19" t="s">
         <v>39</v>
-      </c>
-      <c r="D6" s="19" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" s="22">
         <v>1</v>
       </c>
       <c r="C7" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="19" t="s">
         <v>42</v>
-      </c>
-      <c r="D7" s="19" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B8" s="22">
         <v>1</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B9" s="23">
         <v>0.5</v>
       </c>
       <c r="C9" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="D9" s="19" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B10" s="23">
         <v>1.5</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B11" s="23">
         <v>1.2</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B12" s="21">
         <v>1</v>
       </c>
       <c r="C12" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="19" t="s">
         <v>54</v>
-      </c>
-      <c r="D12" s="19" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="19" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B13" s="22">
         <v>0.3</v>
       </c>
       <c r="C13" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" s="19" t="s">
         <v>57</v>
-      </c>
-      <c r="D13" s="19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -11657,88 +11657,88 @@
         <v>5</v>
       </c>
       <c r="B16" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>60</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A17" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B17" s="20">
         <v>0</v>
       </c>
       <c r="C17" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="D17" s="19" t="s">
         <v>63</v>
-      </c>
-      <c r="D17" s="19" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A18" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B18" s="20">
         <v>0</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A19" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B19" s="20">
         <v>0</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A20" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B20" s="20">
         <v>0</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A21" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B21" s="20">
         <v>0</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="82" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B23" s="83"/>
       <c r="C23" s="83"/>
@@ -11746,7 +11746,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
@@ -11754,18 +11754,18 @@
         <v>5</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B27" s="20">
         <v>0</v>
@@ -11779,7 +11779,7 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B28" s="20">
         <v>0</v>
@@ -11793,7 +11793,7 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B29" s="20">
         <v>0</v>
@@ -11807,7 +11807,7 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B30" s="20">
         <v>0</v>
@@ -11821,7 +11821,7 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B31" s="20">
         <v>0</v>
@@ -11834,12 +11834,12 @@
       </c>
     </row>
     <row r="32" spans="1:4" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="86" t="s">
-        <v>232</v>
-      </c>
-      <c r="B32" s="85"/>
-      <c r="C32" s="85"/>
-      <c r="D32" s="85"/>
+      <c r="A32" s="85" t="s">
+        <v>230</v>
+      </c>
+      <c r="B32" s="86"/>
+      <c r="C32" s="86"/>
+      <c r="D32" s="86"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -11872,12 +11872,12 @@
   <sheetData>
     <row r="1" spans="1:20" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:20" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -11885,61 +11885,61 @@
         <v>5</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>79</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>80</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H4" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="I4" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="J4" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="K4" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="L4" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="L4" s="5" t="s">
+      <c r="M4" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="M4" s="5" t="s">
+      <c r="N4" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="N4" s="5" t="s">
+      <c r="O4" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="O4" s="5" t="s">
+      <c r="P4" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="P4" s="5" t="s">
+      <c r="Q4" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="Q4" s="5" t="s">
+      <c r="R4" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="R4" s="5" t="s">
+      <c r="S4" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="S4" s="5" t="s">
+      <c r="T4" s="5" t="s">
         <v>92</v>
-      </c>
-      <c r="T4" s="5" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.3">
@@ -12354,12 +12354,12 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:20" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -12698,12 +12698,12 @@
   <sheetData>
     <row r="1" spans="1:10" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -12711,36 +12711,36 @@
         <v>5</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="F4" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="G4" s="5" t="s">
+      <c r="H4" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="I4" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="J4" s="5" t="s">
         <v>104</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B5" s="33">
         <f>COUNT(Data_Monthly!$G$2:$G$25)</f>
@@ -12781,7 +12781,7 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B6" s="33">
         <f>COUNT(Data_Monthly!$G$26:$G$49)</f>
@@ -12822,7 +12822,7 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B7" s="33">
         <f>IF(Assumptions!$B$12=1,COUNT(Data_Monthly!$G$50:$G$69),COUNT(Data_Monthly!$G$50:$G$73))</f>
@@ -12863,7 +12863,7 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B8" s="33">
         <f>COUNT(Data_Monthly!$G$74:$G$97)</f>
@@ -12904,7 +12904,7 @@
     </row>
     <row r="10" spans="1:10" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="82" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B10" s="83"/>
       <c r="C10" s="83"/>
@@ -12944,12 +12944,12 @@
   <sheetData>
     <row r="1" spans="1:11" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -12957,39 +12957,39 @@
         <v>5</v>
       </c>
       <c r="B4" s="61" t="s">
+        <v>108</v>
+      </c>
+      <c r="C4" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="C4" s="61" t="s">
+      <c r="D4" s="61" t="s">
         <v>110</v>
       </c>
-      <c r="D4" s="61" t="s">
+      <c r="E4" s="61" t="s">
         <v>111</v>
       </c>
-      <c r="E4" s="61" t="s">
+      <c r="F4" s="61" t="s">
         <v>112</v>
       </c>
-      <c r="F4" s="61" t="s">
+      <c r="G4" s="61" t="s">
         <v>113</v>
       </c>
-      <c r="G4" s="61" t="s">
+      <c r="H4" s="61" t="s">
         <v>114</v>
       </c>
-      <c r="H4" s="61" t="s">
+      <c r="I4" s="61" t="s">
+        <v>92</v>
+      </c>
+      <c r="J4" s="61" t="s">
         <v>115</v>
       </c>
-      <c r="I4" s="61" t="s">
-        <v>93</v>
-      </c>
-      <c r="J4" s="61" t="s">
+      <c r="K4" s="62" t="s">
         <v>116</v>
-      </c>
-      <c r="K4" s="62" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="58" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B5" s="10">
         <f>SUMIFS(Data_Monthly!$C$2:$C$97,Data_Monthly!$A$2:$A$97,A5,Data_Monthly!$E$2:$E$97,1)</f>
@@ -13033,7 +13033,7 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="58" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B6" s="10">
         <f>SUMIFS(Data_Monthly!$C$2:$C$97,Data_Monthly!$A$2:$A$97,A6,Data_Monthly!$E$2:$E$97,1)</f>
@@ -13077,7 +13077,7 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="58" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B7" s="10">
         <f>SUMIFS(Data_Monthly!$C$2:$C$97,Data_Monthly!$A$2:$A$97,A7,Data_Monthly!$E$2:$E$97,1)</f>
@@ -13121,7 +13121,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="63" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B8" s="64">
         <f>SUMIFS(Data_Monthly!$C$2:$C$97,Data_Monthly!$A$2:$A$97,A8,Data_Monthly!$E$2:$E$97,1)</f>
@@ -13201,7 +13201,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="19" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B11" s="10">
         <f>B9*Assumptions!B7</f>
@@ -13210,7 +13210,7 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="19" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B12" s="10">
         <f>E9</f>
@@ -13219,7 +13219,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="19" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B13" s="10">
         <f>J9-B9</f>
@@ -13228,7 +13228,7 @@
     </row>
     <row r="14" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A14" s="41" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B14" s="16">
         <f>K9-E9</f>
@@ -13237,7 +13237,7 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="41" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B15" s="13">
         <f>B14-B13</f>
@@ -13246,7 +13246,7 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B16" s="15" t="str">
         <f>IF(E9&lt;=B11+0.005,"OK","OVER BUDGET")</f>
@@ -13255,7 +13255,7 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="19" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B17" s="15" t="str">
         <f>IF(SUMPRODUCT((E5:E8&lt;C5:C8-0.005)+(E5:E8&gt;D5:D8+0.005))=0,"OK","OUTSIDE LIMITS")</f>
@@ -13264,7 +13264,7 @@
     </row>
     <row r="19" spans="1:11" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="82" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B19" s="83"/>
       <c r="C19" s="83"/>
@@ -13310,58 +13310,58 @@
   <sheetData>
     <row r="1" spans="1:12" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="60" t="s">
+        <v>127</v>
+      </c>
+      <c r="B4" s="61" t="s">
         <v>128</v>
       </c>
-      <c r="B4" s="61" t="s">
+      <c r="C4" s="61" t="s">
+        <v>117</v>
+      </c>
+      <c r="D4" s="61" t="s">
         <v>129</v>
       </c>
-      <c r="C4" s="61" t="s">
-        <v>118</v>
-      </c>
-      <c r="D4" s="61" t="s">
+      <c r="E4" s="61" t="s">
         <v>130</v>
       </c>
-      <c r="E4" s="61" t="s">
+      <c r="F4" s="61" t="s">
         <v>131</v>
       </c>
-      <c r="F4" s="61" t="s">
+      <c r="G4" s="61" t="s">
         <v>132</v>
       </c>
-      <c r="G4" s="61" t="s">
+      <c r="H4" s="61" t="s">
         <v>133</v>
       </c>
-      <c r="H4" s="61" t="s">
+      <c r="I4" s="61" t="s">
         <v>134</v>
       </c>
-      <c r="I4" s="61" t="s">
+      <c r="J4" s="61" t="s">
         <v>135</v>
       </c>
-      <c r="J4" s="61" t="s">
+      <c r="K4" s="61" t="s">
+        <v>119</v>
+      </c>
+      <c r="L4" s="62" t="s">
         <v>136</v>
-      </c>
-      <c r="K4" s="61" t="s">
-        <v>120</v>
-      </c>
-      <c r="L4" s="62" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="70" t="s">
+        <v>137</v>
+      </c>
+      <c r="B5" s="19" t="s">
         <v>138</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>139</v>
       </c>
       <c r="C5" s="10">
         <v>28603</v>
@@ -13398,10 +13398,10 @@
     </row>
     <row r="6" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="70" t="s">
+        <v>139</v>
+      </c>
+      <c r="B6" s="19" t="s">
         <v>140</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>141</v>
       </c>
       <c r="C6" s="10">
         <v>22882</v>
@@ -13438,10 +13438,10 @@
     </row>
     <row r="7" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="70" t="s">
+        <v>141</v>
+      </c>
+      <c r="B7" s="19" t="s">
         <v>142</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>143</v>
       </c>
       <c r="C7" s="10">
         <v>34323</v>
@@ -13478,10 +13478,10 @@
     </row>
     <row r="8" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="70" t="s">
+        <v>143</v>
+      </c>
+      <c r="B8" s="19" t="s">
         <v>144</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>145</v>
       </c>
       <c r="C8" s="10">
         <v>28603</v>
@@ -13518,10 +13518,10 @@
     </row>
     <row r="9" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="70" t="s">
+        <v>145</v>
+      </c>
+      <c r="B9" s="19" t="s">
         <v>146</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>147</v>
       </c>
       <c r="C9" s="10">
         <v>28603</v>
@@ -13558,10 +13558,10 @@
     </row>
     <row r="10" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="70" t="s">
+        <v>147</v>
+      </c>
+      <c r="B10" s="19" t="s">
         <v>148</v>
-      </c>
-      <c r="B10" s="19" t="s">
-        <v>149</v>
       </c>
       <c r="C10" s="10">
         <v>28603</v>
@@ -13598,10 +13598,10 @@
     </row>
     <row r="11" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="70" t="s">
+        <v>149</v>
+      </c>
+      <c r="B11" s="19" t="s">
         <v>150</v>
-      </c>
-      <c r="B11" s="19" t="s">
-        <v>151</v>
       </c>
       <c r="C11" s="10">
         <v>28603</v>
@@ -13638,10 +13638,10 @@
     </row>
     <row r="12" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="72" t="s">
+        <v>151</v>
+      </c>
+      <c r="B12" s="73" t="s">
         <v>152</v>
-      </c>
-      <c r="B12" s="73" t="s">
-        <v>153</v>
       </c>
       <c r="C12" s="64">
         <v>28603</v>
@@ -13678,12 +13678,12 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="82" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B15" s="83"/>
       <c r="C15" s="83"/>
@@ -13720,67 +13720,67 @@
   <sheetData>
     <row r="1" spans="1:15" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4" spans="1:15" s="81" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A4" s="60" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B4" s="61" t="s">
+        <v>233</v>
+      </c>
+      <c r="C4" s="61" t="s">
+        <v>234</v>
+      </c>
+      <c r="D4" s="61" t="s">
         <v>235</v>
       </c>
-      <c r="C4" s="61" t="s">
+      <c r="E4" s="61" t="s">
         <v>236</v>
       </c>
-      <c r="D4" s="61" t="s">
+      <c r="F4" s="61" t="s">
         <v>237</v>
       </c>
-      <c r="E4" s="61" t="s">
-        <v>238</v>
-      </c>
-      <c r="F4" s="61" t="s">
-        <v>239</v>
-      </c>
       <c r="G4" s="61" t="s">
+        <v>129</v>
+      </c>
+      <c r="H4" s="61" t="s">
         <v>130</v>
       </c>
-      <c r="H4" s="61" t="s">
+      <c r="I4" s="61" t="s">
         <v>131</v>
       </c>
-      <c r="I4" s="61" t="s">
+      <c r="J4" s="61" t="s">
         <v>132</v>
       </c>
-      <c r="J4" s="61" t="s">
+      <c r="K4" s="61" t="s">
         <v>133</v>
       </c>
-      <c r="K4" s="61" t="s">
+      <c r="L4" s="62" t="s">
         <v>134</v>
       </c>
-      <c r="L4" s="62" t="s">
+      <c r="M4" s="60" t="s">
         <v>135</v>
       </c>
-      <c r="M4" s="60" t="s">
+      <c r="N4" s="61" t="s">
+        <v>119</v>
+      </c>
+      <c r="O4" s="61" t="s">
         <v>136</v>
-      </c>
-      <c r="N4" s="61" t="s">
-        <v>120</v>
-      </c>
-      <c r="O4" s="61" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="70" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C5" s="77">
         <v>0</v>
@@ -13826,10 +13826,10 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="70" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C6" s="77">
         <v>-220.92</v>
@@ -13875,10 +13875,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="70" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C7" s="77">
         <v>206.55</v>
@@ -13924,10 +13924,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="70" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C8" s="77">
         <v>206.55</v>
@@ -13973,10 +13973,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="70" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C9" s="77">
         <v>-220.92</v>
@@ -14021,23 +14021,23 @@
       </c>
     </row>
     <row r="11" spans="1:15" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="88" t="s">
-        <v>250</v>
-      </c>
-      <c r="B11" s="87"/>
-      <c r="C11" s="87"/>
-      <c r="D11" s="87"/>
-      <c r="E11" s="87"/>
-      <c r="F11" s="87"/>
-      <c r="G11" s="87"/>
-      <c r="H11" s="87"/>
-      <c r="I11" s="87"/>
-      <c r="J11" s="87"/>
-      <c r="K11" s="87"/>
-      <c r="L11" s="87"/>
-      <c r="M11" s="87"/>
-      <c r="N11" s="87"/>
-      <c r="O11" s="87"/>
+      <c r="A11" s="87" t="s">
+        <v>248</v>
+      </c>
+      <c r="B11" s="88"/>
+      <c r="C11" s="88"/>
+      <c r="D11" s="88"/>
+      <c r="E11" s="88"/>
+      <c r="F11" s="88"/>
+      <c r="G11" s="88"/>
+      <c r="H11" s="88"/>
+      <c r="I11" s="88"/>
+      <c r="J11" s="88"/>
+      <c r="K11" s="88"/>
+      <c r="L11" s="88"/>
+      <c r="M11" s="88"/>
+      <c r="N11" s="88"/>
+      <c r="O11" s="88"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Remove empty sheets from the Excel model, update the summary wording and rebuild the Excel walkthrough with the LTV scenarios
</commit_message>
<xml_diff>
--- a/excel/budget_model.xlsx
+++ b/excel/budget_model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40576ae3754c8ac9/Υπολογιστής/Ο Φάκελός μου/Data analyst projects/FinTech Customer Acquisition and Profitability Analysis/FinTech-Customer-Acquisition-and-Profitability-Analysis/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3988" documentId="8_{DA684D4A-D9C9-4D3B-8B67-0B4778129DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{980DA29E-DB2B-49DD-95AD-9A9745B27369}"/>
+  <xr:revisionPtr revIDLastSave="3992" documentId="8_{DA684D4A-D9C9-4D3B-8B67-0B4778129DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22749384-8626-4397-BF49-9B9ED76FDA3F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,15 +20,11 @@
     <sheet name="Optimizer" sheetId="5" r:id="rId5"/>
     <sheet name="Scenarios" sheetId="6" r:id="rId6"/>
     <sheet name="LTV_Scenarios" sheetId="18" r:id="rId7"/>
-    <sheet name="Sheet4" sheetId="17" r:id="rId8"/>
-    <sheet name="Sheet3" sheetId="16" r:id="rId9"/>
-    <sheet name="Sheet2" sheetId="15" r:id="rId10"/>
-    <sheet name="Sheet1" sheetId="14" r:id="rId11"/>
-    <sheet name="Pivot_Tables" sheetId="12" r:id="rId12"/>
-    <sheet name="Notes" sheetId="7" r:id="rId13"/>
-    <sheet name="Data_Scorecard" sheetId="8" r:id="rId14"/>
-    <sheet name="Data_Monthly" sheetId="9" r:id="rId15"/>
-    <sheet name="Data_Curve" sheetId="10" r:id="rId16"/>
+    <sheet name="Pivot_Tables" sheetId="12" r:id="rId8"/>
+    <sheet name="Notes" sheetId="7" r:id="rId9"/>
+    <sheet name="Data_Scorecard" sheetId="8" r:id="rId10"/>
+    <sheet name="Data_Monthly" sheetId="9" r:id="rId11"/>
+    <sheet name="Data_Curve" sheetId="10" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="solver_adj" localSheetId="4" hidden="1">Optimizer!$E$5:$E$8</definedName>
@@ -54,7 +50,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId17"/>
+    <pivotCache cacheId="0" r:id="rId13"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -6408,875 +6404,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D41B753-3D14-4CD8-A6D6-4EDEC0B396DF}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02FD9BB6-92B3-41DA-B0A3-8137671C795C}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C01AF9F-AE8A-4B2F-97D1-ABA6C3D76678}">
-  <dimension ref="A1:F50"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="16.77734375" style="48" customWidth="1"/>
-    <col min="2" max="7" width="12.77734375" style="48" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="48"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="51" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="50" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="56" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="52" t="s">
-        <v>222</v>
-      </c>
-      <c r="B5" s="52" t="s">
-        <v>213</v>
-      </c>
-      <c r="C5"/>
-      <c r="D5"/>
-      <c r="E5"/>
-      <c r="F5"/>
-    </row>
-    <row r="6" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="52" t="s">
-        <v>211</v>
-      </c>
-      <c r="B6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C6" t="s">
-        <v>66</v>
-      </c>
-      <c r="D6" t="s">
-        <v>68</v>
-      </c>
-      <c r="E6" t="s">
-        <v>70</v>
-      </c>
-      <c r="F6" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="53" t="s">
-        <v>214</v>
-      </c>
-      <c r="B7" s="54">
-        <v>3700.24</v>
-      </c>
-      <c r="C7" s="54">
-        <v>5445.75</v>
-      </c>
-      <c r="D7" s="54">
-        <v>8042.77</v>
-      </c>
-      <c r="E7" s="54">
-        <v>1340.53</v>
-      </c>
-      <c r="F7" s="54">
-        <v>18529.29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="53" t="s">
-        <v>215</v>
-      </c>
-      <c r="B8" s="54">
-        <v>2219.08</v>
-      </c>
-      <c r="C8" s="54">
-        <v>4812.82</v>
-      </c>
-      <c r="D8" s="54">
-        <v>6017.4</v>
-      </c>
-      <c r="E8" s="54">
-        <v>979.58999999999992</v>
-      </c>
-      <c r="F8" s="54">
-        <v>14028.89</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="53" t="s">
-        <v>216</v>
-      </c>
-      <c r="B9" s="54">
-        <v>2419.5199999999995</v>
-      </c>
-      <c r="C9" s="54">
-        <v>5129.18</v>
-      </c>
-      <c r="D9" s="54">
-        <v>6144.2900000000009</v>
-      </c>
-      <c r="E9" s="54">
-        <v>946.43000000000006</v>
-      </c>
-      <c r="F9" s="54">
-        <v>14639.420000000002</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="53" t="s">
-        <v>217</v>
-      </c>
-      <c r="B10" s="54">
-        <v>2452.1099999999997</v>
-      </c>
-      <c r="C10" s="54">
-        <v>4997</v>
-      </c>
-      <c r="D10" s="54">
-        <v>6065.59</v>
-      </c>
-      <c r="E10" s="54">
-        <v>1027.5700000000002</v>
-      </c>
-      <c r="F10" s="54">
-        <v>14542.27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A11" s="53" t="s">
-        <v>218</v>
-      </c>
-      <c r="B11" s="54">
-        <v>4148.6100000000006</v>
-      </c>
-      <c r="C11" s="54">
-        <v>7611.43</v>
-      </c>
-      <c r="D11" s="54">
-        <v>11317.44</v>
-      </c>
-      <c r="E11" s="54">
-        <v>1195.72</v>
-      </c>
-      <c r="F11" s="54">
-        <v>24273.200000000004</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="53" t="s">
-        <v>219</v>
-      </c>
-      <c r="B12" s="54">
-        <v>2849.87</v>
-      </c>
-      <c r="C12" s="54">
-        <v>6257.49</v>
-      </c>
-      <c r="D12" s="54">
-        <v>6411.41</v>
-      </c>
-      <c r="E12" s="54">
-        <v>988.06</v>
-      </c>
-      <c r="F12" s="54">
-        <v>16506.830000000002</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="53" t="s">
-        <v>220</v>
-      </c>
-      <c r="B13" s="54">
-        <v>2771.6800000000003</v>
-      </c>
-      <c r="C13" s="54">
-        <v>6052.7400000000007</v>
-      </c>
-      <c r="D13" s="54">
-        <v>10944.369999999999</v>
-      </c>
-      <c r="E13" s="54">
-        <v>1159.55</v>
-      </c>
-      <c r="F13" s="54">
-        <v>20928.34</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="53" t="s">
-        <v>221</v>
-      </c>
-      <c r="B14" s="54">
-        <v>3116.48</v>
-      </c>
-      <c r="C14" s="54">
-        <v>5374.79</v>
-      </c>
-      <c r="D14" s="54">
-        <v>19030.080000000002</v>
-      </c>
-      <c r="E14" s="54">
-        <v>1081.3399999999999</v>
-      </c>
-      <c r="F14" s="54">
-        <v>28602.690000000002</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="53" t="s">
-        <v>212</v>
-      </c>
-      <c r="B15" s="54">
-        <v>23677.59</v>
-      </c>
-      <c r="C15" s="54">
-        <v>45681.2</v>
-      </c>
-      <c r="D15" s="54">
-        <v>73973.349999999991</v>
-      </c>
-      <c r="E15" s="54">
-        <v>8718.7900000000009</v>
-      </c>
-      <c r="F15" s="54">
-        <v>152050.93</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A16"/>
-      <c r="B16"/>
-      <c r="C16"/>
-    </row>
-    <row r="17" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17"/>
-      <c r="B17"/>
-      <c r="C17"/>
-    </row>
-    <row r="18" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="57" t="s">
-        <v>134</v>
-      </c>
-      <c r="B18"/>
-      <c r="C18"/>
-    </row>
-    <row r="19" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="52" t="s">
-        <v>223</v>
-      </c>
-      <c r="B19" s="52" t="s">
-        <v>213</v>
-      </c>
-      <c r="C19"/>
-      <c r="D19"/>
-      <c r="E19"/>
-      <c r="F19"/>
-    </row>
-    <row r="20" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="52" t="s">
-        <v>211</v>
-      </c>
-      <c r="B20" t="s">
-        <v>61</v>
-      </c>
-      <c r="C20" t="s">
-        <v>66</v>
-      </c>
-      <c r="D20" t="s">
-        <v>68</v>
-      </c>
-      <c r="E20" t="s">
-        <v>70</v>
-      </c>
-      <c r="F20" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="53" t="s">
-        <v>214</v>
-      </c>
-      <c r="B21" s="54">
-        <v>97.3</v>
-      </c>
-      <c r="C21" s="54">
-        <v>230.52</v>
-      </c>
-      <c r="D21" s="54">
-        <v>115.52000000000001</v>
-      </c>
-      <c r="E21" s="54">
-        <v>111.77000000000001</v>
-      </c>
-      <c r="F21" s="54">
-        <v>555.11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="53" t="s">
-        <v>215</v>
-      </c>
-      <c r="B22" s="54">
-        <v>96.259999999999991</v>
-      </c>
-      <c r="C22" s="54">
-        <v>211.82</v>
-      </c>
-      <c r="D22" s="54">
-        <v>95.66</v>
-      </c>
-      <c r="E22" s="54">
-        <v>116.5</v>
-      </c>
-      <c r="F22" s="54">
-        <v>520.24</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="53" t="s">
-        <v>216</v>
-      </c>
-      <c r="B23" s="54">
-        <v>90.740000000000009</v>
-      </c>
-      <c r="C23" s="54">
-        <v>227.65</v>
-      </c>
-      <c r="D23" s="54">
-        <v>113.56</v>
-      </c>
-      <c r="E23" s="54">
-        <v>98.47</v>
-      </c>
-      <c r="F23" s="54">
-        <v>530.41999999999996</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A24" s="53" t="s">
-        <v>217</v>
-      </c>
-      <c r="B24" s="54">
-        <v>85.22999999999999</v>
-      </c>
-      <c r="C24" s="54">
-        <v>202.23000000000002</v>
-      </c>
-      <c r="D24" s="54">
-        <v>129.5</v>
-      </c>
-      <c r="E24" s="54">
-        <v>104.87</v>
-      </c>
-      <c r="F24" s="54">
-        <v>521.83000000000004</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="53" t="s">
-        <v>218</v>
-      </c>
-      <c r="B25" s="54">
-        <v>140.46</v>
-      </c>
-      <c r="C25" s="54">
-        <v>268.7</v>
-      </c>
-      <c r="D25" s="54">
-        <v>159.36000000000001</v>
-      </c>
-      <c r="E25" s="54">
-        <v>109.36999999999999</v>
-      </c>
-      <c r="F25" s="54">
-        <v>677.89</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="53" t="s">
-        <v>219</v>
-      </c>
-      <c r="B26" s="54">
-        <v>109.84</v>
-      </c>
-      <c r="C26" s="54">
-        <v>267.16000000000003</v>
-      </c>
-      <c r="D26" s="54">
-        <v>126.93</v>
-      </c>
-      <c r="E26" s="54">
-        <v>100.7</v>
-      </c>
-      <c r="F26" s="54">
-        <v>604.63</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A27" s="53" t="s">
-        <v>220</v>
-      </c>
-      <c r="B27" s="54">
-        <v>113.63</v>
-      </c>
-      <c r="C27" s="54">
-        <v>261.97000000000003</v>
-      </c>
-      <c r="D27" s="54">
-        <v>120.43</v>
-      </c>
-      <c r="E27" s="54">
-        <v>111.67</v>
-      </c>
-      <c r="F27" s="54">
-        <v>607.70000000000005</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A28" s="53" t="s">
-        <v>221</v>
-      </c>
-      <c r="B28" s="54">
-        <v>115.53999999999999</v>
-      </c>
-      <c r="C28" s="54">
-        <v>222.13</v>
-      </c>
-      <c r="D28" s="54">
-        <v>120.43</v>
-      </c>
-      <c r="E28" s="54">
-        <v>109.13999999999999</v>
-      </c>
-      <c r="F28" s="54">
-        <v>567.24</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A29" s="53" t="s">
-        <v>212</v>
-      </c>
-      <c r="B29" s="54">
-        <v>849</v>
-      </c>
-      <c r="C29" s="54">
-        <v>1892.1800000000003</v>
-      </c>
-      <c r="D29" s="54">
-        <v>981.3900000000001</v>
-      </c>
-      <c r="E29" s="54">
-        <v>862.49</v>
-      </c>
-      <c r="F29" s="54">
-        <v>4585.0599999999995</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A30"/>
-      <c r="B30"/>
-      <c r="C30"/>
-    </row>
-    <row r="31" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A31"/>
-      <c r="B31"/>
-      <c r="C31"/>
-    </row>
-    <row r="32" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A32" s="57" t="s">
-        <v>224</v>
-      </c>
-      <c r="B32"/>
-      <c r="C32"/>
-    </row>
-    <row r="33" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A33" s="52" t="s">
-        <v>225</v>
-      </c>
-      <c r="B33" s="52" t="s">
-        <v>213</v>
-      </c>
-      <c r="C33"/>
-      <c r="D33"/>
-      <c r="E33"/>
-      <c r="F33"/>
-    </row>
-    <row r="34" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A34" s="52" t="s">
-        <v>211</v>
-      </c>
-      <c r="B34" t="s">
-        <v>61</v>
-      </c>
-      <c r="C34" t="s">
-        <v>66</v>
-      </c>
-      <c r="D34" t="s">
-        <v>68</v>
-      </c>
-      <c r="E34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F34" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A35" s="53" t="s">
-        <v>214</v>
-      </c>
-      <c r="B35" s="55">
-        <v>38.029188078108938</v>
-      </c>
-      <c r="C35" s="55">
-        <v>23.623763664757938</v>
-      </c>
-      <c r="D35" s="55">
-        <v>69.62231648199446</v>
-      </c>
-      <c r="E35" s="55">
-        <v>11.993647669320925</v>
-      </c>
-      <c r="F35" s="55">
-        <v>33.379492352866997</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A36" s="53" t="s">
-        <v>215</v>
-      </c>
-      <c r="B36" s="55">
-        <v>23.05298150841471</v>
-      </c>
-      <c r="C36" s="55">
-        <v>22.721272778774431</v>
-      </c>
-      <c r="D36" s="55">
-        <v>62.904035124398909</v>
-      </c>
-      <c r="E36" s="55">
-        <v>8.4084978540772521</v>
-      </c>
-      <c r="F36" s="55">
-        <v>26.966188682146701</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A37" s="53" t="s">
-        <v>216</v>
-      </c>
-      <c r="B37" s="55">
-        <v>26.664315627066337</v>
-      </c>
-      <c r="C37" s="55">
-        <v>22.530990555677576</v>
-      </c>
-      <c r="D37" s="55">
-        <v>54.106111306798176</v>
-      </c>
-      <c r="E37" s="55">
-        <v>9.6113537117903931</v>
-      </c>
-      <c r="F37" s="55">
-        <v>27.599675728667844</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A38" s="53" t="s">
-        <v>217</v>
-      </c>
-      <c r="B38" s="55">
-        <v>28.770503343892994</v>
-      </c>
-      <c r="C38" s="55">
-        <v>24.709489195470503</v>
-      </c>
-      <c r="D38" s="55">
-        <v>46.838532818532819</v>
-      </c>
-      <c r="E38" s="55">
-        <v>9.7985124439782592</v>
-      </c>
-      <c r="F38" s="55">
-        <v>27.867830519517845</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A39" s="53" t="s">
-        <v>218</v>
-      </c>
-      <c r="B39" s="55">
-        <v>29.535882101665958</v>
-      </c>
-      <c r="C39" s="55">
-        <v>28.326870115370305</v>
-      </c>
-      <c r="D39" s="55">
-        <v>71.018072289156621</v>
-      </c>
-      <c r="E39" s="55">
-        <v>10.932796927859561</v>
-      </c>
-      <c r="F39" s="55">
-        <v>35.80698933455281</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A40" s="53" t="s">
-        <v>219</v>
-      </c>
-      <c r="B40" s="55">
-        <v>25.945648215586306</v>
-      </c>
-      <c r="C40" s="55">
-        <v>23.422256325797271</v>
-      </c>
-      <c r="D40" s="55">
-        <v>50.511384227526982</v>
-      </c>
-      <c r="E40" s="55">
-        <v>9.8119165839126108</v>
-      </c>
-      <c r="F40" s="55">
-        <v>27.300712832641441</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A41" s="53" t="s">
-        <v>220</v>
-      </c>
-      <c r="B41" s="55">
-        <v>24.392149960397784</v>
-      </c>
-      <c r="C41" s="55">
-        <v>23.104706645799137</v>
-      </c>
-      <c r="D41" s="55">
-        <v>90.877439176284966</v>
-      </c>
-      <c r="E41" s="55">
-        <v>10.383719888958538</v>
-      </c>
-      <c r="F41" s="55">
-        <v>34.438604574625636</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A42" s="53" t="s">
-        <v>221</v>
-      </c>
-      <c r="B42" s="55">
-        <v>26.973169465120307</v>
-      </c>
-      <c r="C42" s="55">
-        <v>24.196596587583848</v>
-      </c>
-      <c r="D42" s="55">
-        <v>158.01776965872293</v>
-      </c>
-      <c r="E42" s="55">
-        <v>9.907824812167858</v>
-      </c>
-      <c r="F42" s="55">
-        <v>50.424317749100915</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A43" s="53" t="s">
-        <v>212</v>
-      </c>
-      <c r="B43" s="55">
-        <v>27.888798586572442</v>
-      </c>
-      <c r="C43" s="55">
-        <v>24.142100645815944</v>
-      </c>
-      <c r="D43" s="55">
-        <v>75.376099206227906</v>
-      </c>
-      <c r="E43" s="55">
-        <v>10.108859233150529</v>
-      </c>
-      <c r="F43" s="55">
-        <v>33.162255237663196</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A44"/>
-      <c r="B44"/>
-      <c r="C44"/>
-    </row>
-    <row r="45" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A45"/>
-      <c r="B45"/>
-      <c r="C45"/>
-    </row>
-    <row r="46" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A46"/>
-      <c r="B46"/>
-      <c r="C46"/>
-    </row>
-    <row r="47" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A47"/>
-      <c r="B47"/>
-      <c r="C47"/>
-    </row>
-    <row r="48" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A48"/>
-      <c r="B48"/>
-      <c r="C48"/>
-    </row>
-    <row r="49" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A49"/>
-      <c r="B49"/>
-      <c r="C49"/>
-    </row>
-    <row r="50" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A50"/>
-      <c r="B50"/>
-      <c r="C50"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId4"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="120" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="41" t="s">
-        <v>156</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="41" t="s">
-        <v>158</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="41" t="s">
-        <v>160</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="41" t="s">
-        <v>162</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="41" t="s">
-        <v>164</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="41" t="s">
-        <v>166</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="41" t="s">
-        <v>167</v>
-      </c>
-      <c r="B10" s="19" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="41" t="s">
-        <v>169</v>
-      </c>
-      <c r="B11" s="19" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="41" t="s">
-        <v>171</v>
-      </c>
-      <c r="B12" s="19" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="46" t="s">
-        <v>204</v>
-      </c>
-      <c r="B13" s="47" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="46" t="s">
-        <v>206</v>
-      </c>
-      <c r="B14" s="47" t="s">
-        <v>207</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:Q9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -7599,7 +6726,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:J97"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -10431,7 +9558,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:G61"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -14051,19 +13178,852 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{688C7ABA-8B71-48C7-A456-D4978829B4A9}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C01AF9F-AE8A-4B2F-97D1-ABA6C3D76678}">
+  <dimension ref="A1:F50"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.77734375" style="48" customWidth="1"/>
+    <col min="2" max="7" width="12.77734375" style="48" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="48"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A1" s="51" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="50" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="56" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A5" s="52" t="s">
+        <v>222</v>
+      </c>
+      <c r="B5" s="52" t="s">
+        <v>213</v>
+      </c>
+      <c r="C5"/>
+      <c r="D5"/>
+      <c r="E5"/>
+      <c r="F5"/>
+    </row>
+    <row r="6" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="52" t="s">
+        <v>211</v>
+      </c>
+      <c r="B6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6" t="s">
+        <v>68</v>
+      </c>
+      <c r="E6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F6" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="53" t="s">
+        <v>214</v>
+      </c>
+      <c r="B7" s="54">
+        <v>3700.24</v>
+      </c>
+      <c r="C7" s="54">
+        <v>5445.75</v>
+      </c>
+      <c r="D7" s="54">
+        <v>8042.77</v>
+      </c>
+      <c r="E7" s="54">
+        <v>1340.53</v>
+      </c>
+      <c r="F7" s="54">
+        <v>18529.29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A8" s="53" t="s">
+        <v>215</v>
+      </c>
+      <c r="B8" s="54">
+        <v>2219.08</v>
+      </c>
+      <c r="C8" s="54">
+        <v>4812.82</v>
+      </c>
+      <c r="D8" s="54">
+        <v>6017.4</v>
+      </c>
+      <c r="E8" s="54">
+        <v>979.58999999999992</v>
+      </c>
+      <c r="F8" s="54">
+        <v>14028.89</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="53" t="s">
+        <v>216</v>
+      </c>
+      <c r="B9" s="54">
+        <v>2419.5199999999995</v>
+      </c>
+      <c r="C9" s="54">
+        <v>5129.18</v>
+      </c>
+      <c r="D9" s="54">
+        <v>6144.2900000000009</v>
+      </c>
+      <c r="E9" s="54">
+        <v>946.43000000000006</v>
+      </c>
+      <c r="F9" s="54">
+        <v>14639.420000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A10" s="53" t="s">
+        <v>217</v>
+      </c>
+      <c r="B10" s="54">
+        <v>2452.1099999999997</v>
+      </c>
+      <c r="C10" s="54">
+        <v>4997</v>
+      </c>
+      <c r="D10" s="54">
+        <v>6065.59</v>
+      </c>
+      <c r="E10" s="54">
+        <v>1027.5700000000002</v>
+      </c>
+      <c r="F10" s="54">
+        <v>14542.27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A11" s="53" t="s">
+        <v>218</v>
+      </c>
+      <c r="B11" s="54">
+        <v>4148.6100000000006</v>
+      </c>
+      <c r="C11" s="54">
+        <v>7611.43</v>
+      </c>
+      <c r="D11" s="54">
+        <v>11317.44</v>
+      </c>
+      <c r="E11" s="54">
+        <v>1195.72</v>
+      </c>
+      <c r="F11" s="54">
+        <v>24273.200000000004</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="53" t="s">
+        <v>219</v>
+      </c>
+      <c r="B12" s="54">
+        <v>2849.87</v>
+      </c>
+      <c r="C12" s="54">
+        <v>6257.49</v>
+      </c>
+      <c r="D12" s="54">
+        <v>6411.41</v>
+      </c>
+      <c r="E12" s="54">
+        <v>988.06</v>
+      </c>
+      <c r="F12" s="54">
+        <v>16506.830000000002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A13" s="53" t="s">
+        <v>220</v>
+      </c>
+      <c r="B13" s="54">
+        <v>2771.6800000000003</v>
+      </c>
+      <c r="C13" s="54">
+        <v>6052.7400000000007</v>
+      </c>
+      <c r="D13" s="54">
+        <v>10944.369999999999</v>
+      </c>
+      <c r="E13" s="54">
+        <v>1159.55</v>
+      </c>
+      <c r="F13" s="54">
+        <v>20928.34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A14" s="53" t="s">
+        <v>221</v>
+      </c>
+      <c r="B14" s="54">
+        <v>3116.48</v>
+      </c>
+      <c r="C14" s="54">
+        <v>5374.79</v>
+      </c>
+      <c r="D14" s="54">
+        <v>19030.080000000002</v>
+      </c>
+      <c r="E14" s="54">
+        <v>1081.3399999999999</v>
+      </c>
+      <c r="F14" s="54">
+        <v>28602.690000000002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="53" t="s">
+        <v>212</v>
+      </c>
+      <c r="B15" s="54">
+        <v>23677.59</v>
+      </c>
+      <c r="C15" s="54">
+        <v>45681.2</v>
+      </c>
+      <c r="D15" s="54">
+        <v>73973.349999999991</v>
+      </c>
+      <c r="E15" s="54">
+        <v>8718.7900000000009</v>
+      </c>
+      <c r="F15" s="54">
+        <v>152050.93</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A16"/>
+      <c r="B16"/>
+      <c r="C16"/>
+    </row>
+    <row r="17" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A17"/>
+      <c r="B17"/>
+      <c r="C17"/>
+    </row>
+    <row r="18" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A18" s="57" t="s">
+        <v>134</v>
+      </c>
+      <c r="B18"/>
+      <c r="C18"/>
+    </row>
+    <row r="19" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A19" s="52" t="s">
+        <v>223</v>
+      </c>
+      <c r="B19" s="52" t="s">
+        <v>213</v>
+      </c>
+      <c r="C19"/>
+      <c r="D19"/>
+      <c r="E19"/>
+      <c r="F19"/>
+    </row>
+    <row r="20" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A20" s="52" t="s">
+        <v>211</v>
+      </c>
+      <c r="B20" t="s">
+        <v>61</v>
+      </c>
+      <c r="C20" t="s">
+        <v>66</v>
+      </c>
+      <c r="D20" t="s">
+        <v>68</v>
+      </c>
+      <c r="E20" t="s">
+        <v>70</v>
+      </c>
+      <c r="F20" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="53" t="s">
+        <v>214</v>
+      </c>
+      <c r="B21" s="54">
+        <v>97.3</v>
+      </c>
+      <c r="C21" s="54">
+        <v>230.52</v>
+      </c>
+      <c r="D21" s="54">
+        <v>115.52000000000001</v>
+      </c>
+      <c r="E21" s="54">
+        <v>111.77000000000001</v>
+      </c>
+      <c r="F21" s="54">
+        <v>555.11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A22" s="53" t="s">
+        <v>215</v>
+      </c>
+      <c r="B22" s="54">
+        <v>96.259999999999991</v>
+      </c>
+      <c r="C22" s="54">
+        <v>211.82</v>
+      </c>
+      <c r="D22" s="54">
+        <v>95.66</v>
+      </c>
+      <c r="E22" s="54">
+        <v>116.5</v>
+      </c>
+      <c r="F22" s="54">
+        <v>520.24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A23" s="53" t="s">
+        <v>216</v>
+      </c>
+      <c r="B23" s="54">
+        <v>90.740000000000009</v>
+      </c>
+      <c r="C23" s="54">
+        <v>227.65</v>
+      </c>
+      <c r="D23" s="54">
+        <v>113.56</v>
+      </c>
+      <c r="E23" s="54">
+        <v>98.47</v>
+      </c>
+      <c r="F23" s="54">
+        <v>530.41999999999996</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A24" s="53" t="s">
+        <v>217</v>
+      </c>
+      <c r="B24" s="54">
+        <v>85.22999999999999</v>
+      </c>
+      <c r="C24" s="54">
+        <v>202.23000000000002</v>
+      </c>
+      <c r="D24" s="54">
+        <v>129.5</v>
+      </c>
+      <c r="E24" s="54">
+        <v>104.87</v>
+      </c>
+      <c r="F24" s="54">
+        <v>521.83000000000004</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A25" s="53" t="s">
+        <v>218</v>
+      </c>
+      <c r="B25" s="54">
+        <v>140.46</v>
+      </c>
+      <c r="C25" s="54">
+        <v>268.7</v>
+      </c>
+      <c r="D25" s="54">
+        <v>159.36000000000001</v>
+      </c>
+      <c r="E25" s="54">
+        <v>109.36999999999999</v>
+      </c>
+      <c r="F25" s="54">
+        <v>677.89</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A26" s="53" t="s">
+        <v>219</v>
+      </c>
+      <c r="B26" s="54">
+        <v>109.84</v>
+      </c>
+      <c r="C26" s="54">
+        <v>267.16000000000003</v>
+      </c>
+      <c r="D26" s="54">
+        <v>126.93</v>
+      </c>
+      <c r="E26" s="54">
+        <v>100.7</v>
+      </c>
+      <c r="F26" s="54">
+        <v>604.63</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A27" s="53" t="s">
+        <v>220</v>
+      </c>
+      <c r="B27" s="54">
+        <v>113.63</v>
+      </c>
+      <c r="C27" s="54">
+        <v>261.97000000000003</v>
+      </c>
+      <c r="D27" s="54">
+        <v>120.43</v>
+      </c>
+      <c r="E27" s="54">
+        <v>111.67</v>
+      </c>
+      <c r="F27" s="54">
+        <v>607.70000000000005</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A28" s="53" t="s">
+        <v>221</v>
+      </c>
+      <c r="B28" s="54">
+        <v>115.53999999999999</v>
+      </c>
+      <c r="C28" s="54">
+        <v>222.13</v>
+      </c>
+      <c r="D28" s="54">
+        <v>120.43</v>
+      </c>
+      <c r="E28" s="54">
+        <v>109.13999999999999</v>
+      </c>
+      <c r="F28" s="54">
+        <v>567.24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A29" s="53" t="s">
+        <v>212</v>
+      </c>
+      <c r="B29" s="54">
+        <v>849</v>
+      </c>
+      <c r="C29" s="54">
+        <v>1892.1800000000003</v>
+      </c>
+      <c r="D29" s="54">
+        <v>981.3900000000001</v>
+      </c>
+      <c r="E29" s="54">
+        <v>862.49</v>
+      </c>
+      <c r="F29" s="54">
+        <v>4585.0599999999995</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A30"/>
+      <c r="B30"/>
+      <c r="C30"/>
+    </row>
+    <row r="31" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A31"/>
+      <c r="B31"/>
+      <c r="C31"/>
+    </row>
+    <row r="32" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A32" s="57" t="s">
+        <v>224</v>
+      </c>
+      <c r="B32"/>
+      <c r="C32"/>
+    </row>
+    <row r="33" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A33" s="52" t="s">
+        <v>225</v>
+      </c>
+      <c r="B33" s="52" t="s">
+        <v>213</v>
+      </c>
+      <c r="C33"/>
+      <c r="D33"/>
+      <c r="E33"/>
+      <c r="F33"/>
+    </row>
+    <row r="34" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A34" s="52" t="s">
+        <v>211</v>
+      </c>
+      <c r="B34" t="s">
+        <v>61</v>
+      </c>
+      <c r="C34" t="s">
+        <v>66</v>
+      </c>
+      <c r="D34" t="s">
+        <v>68</v>
+      </c>
+      <c r="E34" t="s">
+        <v>70</v>
+      </c>
+      <c r="F34" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A35" s="53" t="s">
+        <v>214</v>
+      </c>
+      <c r="B35" s="55">
+        <v>38.029188078108938</v>
+      </c>
+      <c r="C35" s="55">
+        <v>23.623763664757938</v>
+      </c>
+      <c r="D35" s="55">
+        <v>69.62231648199446</v>
+      </c>
+      <c r="E35" s="55">
+        <v>11.993647669320925</v>
+      </c>
+      <c r="F35" s="55">
+        <v>33.379492352866997</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A36" s="53" t="s">
+        <v>215</v>
+      </c>
+      <c r="B36" s="55">
+        <v>23.05298150841471</v>
+      </c>
+      <c r="C36" s="55">
+        <v>22.721272778774431</v>
+      </c>
+      <c r="D36" s="55">
+        <v>62.904035124398909</v>
+      </c>
+      <c r="E36" s="55">
+        <v>8.4084978540772521</v>
+      </c>
+      <c r="F36" s="55">
+        <v>26.966188682146701</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A37" s="53" t="s">
+        <v>216</v>
+      </c>
+      <c r="B37" s="55">
+        <v>26.664315627066337</v>
+      </c>
+      <c r="C37" s="55">
+        <v>22.530990555677576</v>
+      </c>
+      <c r="D37" s="55">
+        <v>54.106111306798176</v>
+      </c>
+      <c r="E37" s="55">
+        <v>9.6113537117903931</v>
+      </c>
+      <c r="F37" s="55">
+        <v>27.599675728667844</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A38" s="53" t="s">
+        <v>217</v>
+      </c>
+      <c r="B38" s="55">
+        <v>28.770503343892994</v>
+      </c>
+      <c r="C38" s="55">
+        <v>24.709489195470503</v>
+      </c>
+      <c r="D38" s="55">
+        <v>46.838532818532819</v>
+      </c>
+      <c r="E38" s="55">
+        <v>9.7985124439782592</v>
+      </c>
+      <c r="F38" s="55">
+        <v>27.867830519517845</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A39" s="53" t="s">
+        <v>218</v>
+      </c>
+      <c r="B39" s="55">
+        <v>29.535882101665958</v>
+      </c>
+      <c r="C39" s="55">
+        <v>28.326870115370305</v>
+      </c>
+      <c r="D39" s="55">
+        <v>71.018072289156621</v>
+      </c>
+      <c r="E39" s="55">
+        <v>10.932796927859561</v>
+      </c>
+      <c r="F39" s="55">
+        <v>35.80698933455281</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A40" s="53" t="s">
+        <v>219</v>
+      </c>
+      <c r="B40" s="55">
+        <v>25.945648215586306</v>
+      </c>
+      <c r="C40" s="55">
+        <v>23.422256325797271</v>
+      </c>
+      <c r="D40" s="55">
+        <v>50.511384227526982</v>
+      </c>
+      <c r="E40" s="55">
+        <v>9.8119165839126108</v>
+      </c>
+      <c r="F40" s="55">
+        <v>27.300712832641441</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A41" s="53" t="s">
+        <v>220</v>
+      </c>
+      <c r="B41" s="55">
+        <v>24.392149960397784</v>
+      </c>
+      <c r="C41" s="55">
+        <v>23.104706645799137</v>
+      </c>
+      <c r="D41" s="55">
+        <v>90.877439176284966</v>
+      </c>
+      <c r="E41" s="55">
+        <v>10.383719888958538</v>
+      </c>
+      <c r="F41" s="55">
+        <v>34.438604574625636</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A42" s="53" t="s">
+        <v>221</v>
+      </c>
+      <c r="B42" s="55">
+        <v>26.973169465120307</v>
+      </c>
+      <c r="C42" s="55">
+        <v>24.196596587583848</v>
+      </c>
+      <c r="D42" s="55">
+        <v>158.01776965872293</v>
+      </c>
+      <c r="E42" s="55">
+        <v>9.907824812167858</v>
+      </c>
+      <c r="F42" s="55">
+        <v>50.424317749100915</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A43" s="53" t="s">
+        <v>212</v>
+      </c>
+      <c r="B43" s="55">
+        <v>27.888798586572442</v>
+      </c>
+      <c r="C43" s="55">
+        <v>24.142100645815944</v>
+      </c>
+      <c r="D43" s="55">
+        <v>75.376099206227906</v>
+      </c>
+      <c r="E43" s="55">
+        <v>10.108859233150529</v>
+      </c>
+      <c r="F43" s="55">
+        <v>33.162255237663196</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A44"/>
+      <c r="B44"/>
+      <c r="C44"/>
+    </row>
+    <row r="45" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A45"/>
+      <c r="B45"/>
+      <c r="C45"/>
+    </row>
+    <row r="46" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A46"/>
+      <c r="B46"/>
+      <c r="C46"/>
+    </row>
+    <row r="47" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A47"/>
+      <c r="B47"/>
+      <c r="C47"/>
+    </row>
+    <row r="48" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A48"/>
+      <c r="B48"/>
+      <c r="C48"/>
+    </row>
+    <row r="49" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A49"/>
+      <c r="B49"/>
+      <c r="C49"/>
+    </row>
+    <row r="50" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A50"/>
+      <c r="B50"/>
+      <c r="C50"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId4"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF1ED514-E10E-4E95-8B6A-02C8F94ECDA5}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="120" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="41" t="s">
+        <v>156</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="41" t="s">
+        <v>158</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="41" t="s">
+        <v>160</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="41" t="s">
+        <v>162</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="41" t="s">
+        <v>164</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="41" t="s">
+        <v>166</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="41" t="s">
+        <v>167</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="41" t="s">
+        <v>169</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="61.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="41" t="s">
+        <v>171</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="46" t="s">
+        <v>204</v>
+      </c>
+      <c r="B13" s="47" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="46" t="s">
+        <v>206</v>
+      </c>
+      <c r="B14" s="47" t="s">
+        <v>207</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>